<commit_message>
fix(equipment): standardize Brand & Model, resolve 28 4DEM brand conflicts, and fix EQ-IV-0001
</commit_message>
<xml_diff>
--- a/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
+++ b/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
@@ -478,7 +478,7 @@
         <v>TOUCH32-MiniPC</v>
       </c>
       <c r="K2" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L2" t="str">
         <v>2026-08-19</v>
@@ -525,7 +525,7 @@
         <v>TOUCH32-MiniPC</v>
       </c>
       <c r="K3" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L3" t="str">
         <v>2026-08-19</v>
@@ -572,7 +572,7 @@
         <v>TV-LED-43</v>
       </c>
       <c r="K4" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L4" t="str">
         <v>2026-08-19</v>
@@ -619,7 +619,7 @@
         <v>TV-LED-43</v>
       </c>
       <c r="K5" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L5" t="str">
         <v>2026-08-19</v>
@@ -666,7 +666,7 @@
         <v>TOUCH32</v>
       </c>
       <c r="K6" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L6" t="str">
         <v>2026-08-19</v>
@@ -713,7 +713,7 @@
         <v>TOUCH32</v>
       </c>
       <c r="K7" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L7" t="str">
         <v>2026-08-19</v>
@@ -760,7 +760,7 @@
         <v>touchscreen-65 NC</v>
       </c>
       <c r="K8" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L8" t="str">
         <v>2026-08-19</v>
@@ -807,7 +807,7 @@
         <v>touchscreen-65 NC</v>
       </c>
       <c r="K9" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L9" t="str">
         <v>2026-08-19</v>
@@ -854,7 +854,7 @@
         <v>touchscreen-65 NC</v>
       </c>
       <c r="K10" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L10" t="str">
         <v>2026-08-19</v>
@@ -901,7 +901,7 @@
         <v>touchscreen-65 NC</v>
       </c>
       <c r="K11" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L11" t="str">
         <v>2026-08-19</v>
@@ -948,7 +948,7 @@
         <v>04.4510.08</v>
       </c>
       <c r="K12" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L12" t="str">
         <v>2026-08-19</v>
@@ -995,7 +995,7 @@
         <v>04.4510.08</v>
       </c>
       <c r="K13" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L13" t="str">
         <v>2026-08-19</v>
@@ -1042,7 +1042,7 @@
         <v>04.4510.08</v>
       </c>
       <c r="K14" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L14" t="str">
         <v>2026-08-19</v>
@@ -1089,7 +1089,7 @@
         <v>04.4510.08</v>
       </c>
       <c r="K15" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L15" t="str">
         <v>2026-08-19</v>
@@ -1136,7 +1136,7 @@
         <v>04.4510.08</v>
       </c>
       <c r="K16" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L16" t="str">
         <v>2026-08-19</v>
@@ -1183,7 +1183,7 @@
         <v>DT-R2050</v>
       </c>
       <c r="K17" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L17" t="str">
         <v>2026-08-19</v>
@@ -1230,7 +1230,7 @@
         <v>DT-R2050</v>
       </c>
       <c r="K18" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L18" t="str">
         <v>2026-08-19</v>
@@ -1277,7 +1277,7 @@
         <v>DT-R2050</v>
       </c>
       <c r="K19" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L19" t="str">
         <v>2026-08-19</v>
@@ -1324,7 +1324,7 @@
         <v>DT-R2050</v>
       </c>
       <c r="K20" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L20" t="str">
         <v>2026-08-19</v>
@@ -1371,7 +1371,7 @@
         <v>DT-R2050</v>
       </c>
       <c r="K21" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L21" t="str">
         <v>2026-08-19</v>
@@ -1418,7 +1418,7 @@
         <v>DT-R2050</v>
       </c>
       <c r="K22" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L22" t="str">
         <v>2026-08-19</v>
@@ -1465,7 +1465,7 @@
         <v>DT-R2050</v>
       </c>
       <c r="K23" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L23" t="str">
         <v>2026-08-19</v>
@@ -1512,7 +1512,7 @@
         <v>DT-R2050</v>
       </c>
       <c r="K24" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L24" t="str">
         <v>2026-08-19</v>
@@ -1559,7 +1559,7 @@
         <v>DT-R2050</v>
       </c>
       <c r="K25" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L25" t="str">
         <v>2026-08-19</v>
@@ -1606,7 +1606,7 @@
         <v>DT-R2050</v>
       </c>
       <c r="K26" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L26" t="str">
         <v>2026-08-19</v>
@@ -1653,7 +1653,7 @@
         <v>Efficia DFM100</v>
       </c>
       <c r="K27" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L27" t="str">
         <v>2026-08-19</v>
@@ -1700,7 +1700,7 @@
         <v>Efficia DFM100</v>
       </c>
       <c r="K28" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L28" t="str">
         <v>2026-08-19</v>
@@ -1747,7 +1747,7 @@
         <v>AED 3 Trainer</v>
       </c>
       <c r="K29" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L29" t="str">
         <v>2025-06-28</v>
@@ -1794,7 +1794,7 @@
         <v>AED 3 Trainer</v>
       </c>
       <c r="K30" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L30" t="str">
         <v>2025-06-28</v>
@@ -1841,7 +1841,7 @@
         <v>AED 3 Trainer</v>
       </c>
       <c r="K31" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L31" t="str">
         <v>2026-08-19</v>
@@ -1888,7 +1888,7 @@
         <v>AED 3 Trainer</v>
       </c>
       <c r="K32" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L32" t="str">
         <v>2026-08-19</v>
@@ -1935,7 +1935,7 @@
         <v>AED 3 Trainer</v>
       </c>
       <c r="K33" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L33" t="str">
         <v>2026-08-19</v>
@@ -1982,7 +1982,7 @@
         <v>AED 3 Trainer</v>
       </c>
       <c r="K34" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L34" t="str">
         <v>2026-08-19</v>
@@ -2029,7 +2029,7 @@
         <v>AED 3 Trainer</v>
       </c>
       <c r="K35" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L35" t="str">
         <v>2026-08-19</v>
@@ -2076,7 +2076,7 @@
         <v>DT-FB202H</v>
       </c>
       <c r="K36" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L36" t="str">
         <v>2026-08-19</v>
@@ -2123,7 +2123,7 @@
         <v>DT-FB202H</v>
       </c>
       <c r="K37" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L37" t="str">
         <v>2026-08-19</v>
@@ -2170,7 +2170,7 @@
         <v>LeonardoHF-Bed</v>
       </c>
       <c r="K38" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L38" t="str">
         <v>2026-08-19</v>
@@ -2217,7 +2217,7 @@
         <v>Amoul Man Pro (AMM-P)</v>
       </c>
       <c r="K39" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L39" t="str">
         <v>2025-06-28</v>
@@ -2264,7 +2264,7 @@
         <v>Amoul Man Pro (AMM-P)</v>
       </c>
       <c r="K40" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L40" t="str">
         <v>2025-06-28</v>
@@ -2546,7 +2546,7 @@
         <v>Amoul Man Pro (AMM-P)</v>
       </c>
       <c r="K46" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L46" t="str">
         <v>2026-08-19</v>
@@ -2593,7 +2593,7 @@
         <v>Amoul Man Pro (AMM-P)</v>
       </c>
       <c r="K47" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L47" t="str">
         <v>2026-08-19</v>
@@ -2640,7 +2640,7 @@
         <v>Amoul Man Pro (AMM-P)</v>
       </c>
       <c r="K48" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L48" t="str">
         <v>2026-08-19</v>
@@ -2687,7 +2687,7 @@
         <v>Baby CPR Light-indicator</v>
       </c>
       <c r="K49" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L49" t="str">
         <v>2025-06-28</v>
@@ -2734,7 +2734,7 @@
         <v>Baby CPR Light-indicator</v>
       </c>
       <c r="K50" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L50" t="str">
         <v>2025-06-28</v>
@@ -2781,7 +2781,7 @@
         <v>101-7140-8Y (KERi)</v>
       </c>
       <c r="K51" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L51" t="str">
         <v>2026-08-19</v>
@@ -2828,7 +2828,7 @@
         <v>101-7140-8Y (KERi)</v>
       </c>
       <c r="K52" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L52" t="str">
         <v>2026-08-19</v>
@@ -2875,7 +2875,7 @@
         <v>M155</v>
       </c>
       <c r="K53" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L53" t="str">
         <v>2025-06-28</v>
@@ -2922,7 +2922,7 @@
         <v>M155</v>
       </c>
       <c r="K54" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L54" t="str">
         <v>2026-08-19</v>
@@ -2969,7 +2969,7 @@
         <v>M155</v>
       </c>
       <c r="K55" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L55" t="str">
         <v>2026-08-19</v>
@@ -3016,7 +3016,7 @@
         <v>M155</v>
       </c>
       <c r="K56" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L56" t="str">
         <v>2026-08-19</v>
@@ -3063,7 +3063,7 @@
         <v>M155</v>
       </c>
       <c r="K57" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L57" t="str">
         <v>2026-08-19</v>
@@ -3110,7 +3110,7 @@
         <v>M152</v>
       </c>
       <c r="K58" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L58" t="str">
         <v>2026-08-19</v>
@@ -3157,7 +3157,7 @@
         <v>M152</v>
       </c>
       <c r="K59" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L59" t="str">
         <v>2026-08-19</v>
@@ -3204,7 +3204,7 @@
         <v>M152</v>
       </c>
       <c r="K60" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L60" t="str">
         <v>2026-08-19</v>
@@ -3251,7 +3251,7 @@
         <v>M152</v>
       </c>
       <c r="K61" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L61" t="str">
         <v>2026-08-19</v>
@@ -3298,7 +3298,7 @@
         <v>M152</v>
       </c>
       <c r="K62" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L62" t="str">
         <v>2026-08-19</v>
@@ -3345,7 +3345,7 @@
         <v>LF01174</v>
       </c>
       <c r="K63" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L63" t="str">
         <v>2026-08-19</v>
@@ -3392,7 +3392,7 @@
         <v>LF01174</v>
       </c>
       <c r="K64" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L64" t="str">
         <v>2026-08-19</v>
@@ -3439,7 +3439,7 @@
         <v>LF01174</v>
       </c>
       <c r="K65" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L65" t="str">
         <v>2026-08-19</v>
@@ -3486,7 +3486,7 @@
         <v>LF01174</v>
       </c>
       <c r="K66" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L66" t="str">
         <v>2026-08-19</v>
@@ -3533,7 +3533,7 @@
         <v>LF01174</v>
       </c>
       <c r="K67" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L67" t="str">
         <v>2026-08-19</v>
@@ -3580,7 +3580,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K68" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L68" t="str">
         <v>2025-06-28</v>
@@ -3627,7 +3627,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K69" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L69" t="str">
         <v>2025-06-28</v>
@@ -3674,7 +3674,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K70" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L70" t="str">
         <v>2025-06-28</v>
@@ -3721,7 +3721,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K71" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L71" t="str">
         <v>2026-08-19</v>
@@ -3768,7 +3768,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K72" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L72" t="str">
         <v>2026-08-19</v>
@@ -3815,7 +3815,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K73" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L73" t="str">
         <v>2026-08-19</v>
@@ -3862,7 +3862,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K74" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L74" t="str">
         <v>2026-08-19</v>
@@ -3909,7 +3909,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K75" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L75" t="str">
         <v>2026-08-19</v>
@@ -3956,7 +3956,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K76" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L76" t="str">
         <v>2026-08-19</v>
@@ -4003,7 +4003,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K77" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L77" t="str">
         <v>2026-08-19</v>
@@ -4050,7 +4050,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K78" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L78" t="str">
         <v>2026-08-19</v>
@@ -4097,7 +4097,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K79" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L79" t="str">
         <v>2026-08-19</v>
@@ -4144,7 +4144,7 @@
         <v>P93SPC-S</v>
       </c>
       <c r="K80" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L80" t="str">
         <v>2026-08-19</v>
@@ -4191,7 +4191,7 @@
         <v>40201</v>
       </c>
       <c r="K81" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L81" t="str">
         <v>2025-06-28</v>
@@ -4238,7 +4238,7 @@
         <v>40201</v>
       </c>
       <c r="K82" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L82" t="str">
         <v>2026-08-19</v>
@@ -4285,7 +4285,7 @@
         <v>40201</v>
       </c>
       <c r="K83" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L83" t="str">
         <v>2026-08-19</v>
@@ -4332,7 +4332,7 @@
         <v>40201</v>
       </c>
       <c r="K84" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L84" t="str">
         <v>2026-08-19</v>
@@ -4379,7 +4379,7 @@
         <v>40201</v>
       </c>
       <c r="K85" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L85" t="str">
         <v>2026-08-19</v>
@@ -4426,7 +4426,7 @@
         <v>40201</v>
       </c>
       <c r="K86" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L86" t="str">
         <v>2026-08-19</v>
@@ -4473,7 +4473,7 @@
         <v>P100</v>
       </c>
       <c r="K87" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L87" t="str">
         <v>2026-08-19</v>
@@ -4520,7 +4520,7 @@
         <v>P100</v>
       </c>
       <c r="K88" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L88" t="str">
         <v>2026-08-19</v>
@@ -4567,7 +4567,7 @@
         <v>P100</v>
       </c>
       <c r="K89" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L89" t="str">
         <v>2026-08-19</v>
@@ -4614,7 +4614,7 @@
         <v>P100</v>
       </c>
       <c r="K90" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L90" t="str">
         <v>2026-08-19</v>
@@ -4661,7 +4661,7 @@
         <v>P100</v>
       </c>
       <c r="K91" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L91" t="str">
         <v>2026-08-19</v>
@@ -4708,7 +4708,7 @@
         <v>P101</v>
       </c>
       <c r="K92" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L92" t="str">
         <v>2026-08-19</v>
@@ -4755,7 +4755,7 @@
         <v>P101</v>
       </c>
       <c r="K93" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L93" t="str">
         <v>2026-08-19</v>
@@ -4802,7 +4802,7 @@
         <v>P101</v>
       </c>
       <c r="K94" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L94" t="str">
         <v>2026-08-19</v>
@@ -4849,7 +4849,7 @@
         <v>P101</v>
       </c>
       <c r="K95" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L95" t="str">
         <v>2026-08-19</v>
@@ -4896,7 +4896,7 @@
         <v>LF01034</v>
       </c>
       <c r="K96" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L96" t="str">
         <v>2026-08-19</v>
@@ -4943,7 +4943,7 @@
         <v>LF01034</v>
       </c>
       <c r="K97" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L97" t="str">
         <v>2026-08-19</v>
@@ -4990,7 +4990,7 @@
         <v>LF01034</v>
       </c>
       <c r="K98" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L98" t="str">
         <v>2026-08-19</v>
@@ -5037,7 +5037,7 @@
         <v>LF01034</v>
       </c>
       <c r="K99" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L99" t="str">
         <v>2026-08-19</v>
@@ -5084,7 +5084,7 @@
         <v>LF01043</v>
       </c>
       <c r="K100" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L100" t="str">
         <v>2025-06-28</v>
@@ -5131,7 +5131,7 @@
         <v>LF01043</v>
       </c>
       <c r="K101" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L101" t="str">
         <v>2025-06-28</v>
@@ -5178,7 +5178,7 @@
         <v>LF01043</v>
       </c>
       <c r="K102" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L102" t="str">
         <v>2026-08-19</v>
@@ -5225,7 +5225,7 @@
         <v>LF01043</v>
       </c>
       <c r="K103" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L103" t="str">
         <v>2026-08-19</v>
@@ -5272,7 +5272,7 @@
         <v>LF01043</v>
       </c>
       <c r="K104" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L104" t="str">
         <v>2026-08-19</v>
@@ -5319,7 +5319,7 @@
         <v>LF01043</v>
       </c>
       <c r="K105" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L105" t="str">
         <v>2026-08-19</v>
@@ -5366,7 +5366,7 @@
         <v>LF01043</v>
       </c>
       <c r="K106" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L106" t="str">
         <v>2026-08-19</v>
@@ -5413,7 +5413,7 @@
         <v>LF01043</v>
       </c>
       <c r="K107" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L107" t="str">
         <v>2026-08-19</v>
@@ -5460,7 +5460,7 @@
         <v>LF01043</v>
       </c>
       <c r="K108" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L108" t="str">
         <v>2026-08-19</v>
@@ -5507,7 +5507,7 @@
         <v>LF01043</v>
       </c>
       <c r="K109" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L109" t="str">
         <v>2026-08-19</v>
@@ -5554,7 +5554,7 @@
         <v>LF01043</v>
       </c>
       <c r="K110" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L110" t="str">
         <v>2026-08-19</v>
@@ -5601,7 +5601,7 @@
         <v>LF01043</v>
       </c>
       <c r="K111" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L111" t="str">
         <v>2026-08-19</v>
@@ -5648,7 +5648,7 @@
         <v>718-8804 SAM</v>
       </c>
       <c r="K112" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L112" t="str">
         <v>2026-08-19</v>
@@ -5695,7 +5695,7 @@
         <v>718-8804 SAM</v>
       </c>
       <c r="K113" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L113" t="str">
         <v>2026-08-19</v>
@@ -5742,7 +5742,7 @@
         <v>718-8804 SAM</v>
       </c>
       <c r="K114" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L114" t="str">
         <v>2026-08-19</v>
@@ -5789,7 +5789,7 @@
         <v>718-8804 SAM</v>
       </c>
       <c r="K115" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L115" t="str">
         <v>2026-08-19</v>
@@ -5836,7 +5836,7 @@
         <v>718-8804 SAM</v>
       </c>
       <c r="K116" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L116" t="str">
         <v>2026-08-19</v>
@@ -5883,7 +5883,7 @@
         <v>718-8804 SAM</v>
       </c>
       <c r="K117" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L117" t="str">
         <v>2026-08-19</v>
@@ -5930,7 +5930,7 @@
         <v>718-8804 SAM</v>
       </c>
       <c r="K118" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L118" t="str">
         <v>2026-08-19</v>
@@ -5977,7 +5977,7 @@
         <v>718-8804 SAM</v>
       </c>
       <c r="K119" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L119" t="str">
         <v>2026-08-19</v>
@@ -6024,7 +6024,7 @@
         <v>718-8804 SAM</v>
       </c>
       <c r="K120" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L120" t="str">
         <v>2026-08-19</v>
@@ -6071,7 +6071,7 @@
         <v>718-8804 SAM</v>
       </c>
       <c r="K121" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L121" t="str">
         <v>2026-08-19</v>
@@ -6118,7 +6118,7 @@
         <v>LeonardoHF</v>
       </c>
       <c r="K122" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L122" t="str">
         <v>2026-08-19</v>
@@ -6165,7 +6165,7 @@
         <v>iPad 10.2 Wi-Fi</v>
       </c>
       <c r="K123" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L123" t="str">
         <v>2026-08-19</v>
@@ -6212,7 +6212,7 @@
         <v>iPad 10.2 Wi-Fi</v>
       </c>
       <c r="K124" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L124" t="str">
         <v>2026-08-19</v>
@@ -6259,7 +6259,7 @@
         <v>iPad 10.2 Wi-Fi</v>
       </c>
       <c r="K125" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L125" t="str">
         <v>2026-08-19</v>
@@ -6306,7 +6306,7 @@
         <v>iPad 10.2 Wi-Fi</v>
       </c>
       <c r="K126" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L126" t="str">
         <v>2026-08-19</v>
@@ -6353,7 +6353,7 @@
         <v>iPad 10.2 Wi-Fi</v>
       </c>
       <c r="K127" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L127" t="str">
         <v>2026-08-19</v>
@@ -6400,7 +6400,7 @@
         <v>iPad 10.2 Wi-Fi</v>
       </c>
       <c r="K128" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L128" t="str">
         <v>2026-08-19</v>
@@ -6447,7 +6447,7 @@
         <v>iPad 10.2 Wi-Fi</v>
       </c>
       <c r="K129" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L129" t="str">
         <v>2026-08-19</v>
@@ -6494,7 +6494,7 @@
         <v>iPad 10.2 Wi-Fi</v>
       </c>
       <c r="K130" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L130" t="str">
         <v>2026-08-19</v>
@@ -6541,7 +6541,7 @@
         <v>iPad 10.2 Wi-Fi</v>
       </c>
       <c r="K131" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L131" t="str">
         <v>2026-08-19</v>
@@ -6588,7 +6588,7 @@
         <v>iPad 10.2 Wi-Fi</v>
       </c>
       <c r="K132" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L132" t="str">
         <v>2026-08-19</v>
@@ -6635,7 +6635,7 @@
         <v>BI-30SW-4Y-TH</v>
       </c>
       <c r="K133" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L133" t="str">
         <v>2029-08-19</v>
@@ -6682,7 +6682,7 @@
         <v>เตียงตรวจโรคมาตรฐาน</v>
       </c>
       <c r="K134" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L134" t="str">
         <v>2025-08-01</v>
@@ -6729,7 +6729,7 @@
         <v>CPR Board (CPR-B)</v>
       </c>
       <c r="K135" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L135" t="str">
         <v>2025-06-28</v>
@@ -6776,7 +6776,7 @@
         <v>CPR Board (CPR-B)</v>
       </c>
       <c r="K136" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L136" t="str">
         <v>2026-08-19</v>
@@ -6823,7 +6823,7 @@
         <v>CPR Board (CPR-B)</v>
       </c>
       <c r="K137" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L137" t="str">
         <v>2026-08-19</v>
@@ -6870,7 +6870,7 @@
         <v>CPR Board (CPR-B)</v>
       </c>
       <c r="K138" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L138" t="str">
         <v>2026-08-19</v>
@@ -6917,7 +6917,7 @@
         <v>LF01043</v>
       </c>
       <c r="K139" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L139" t="str">
         <v>2026-08-19</v>
@@ -6964,7 +6964,7 @@
         <v>LF01043</v>
       </c>
       <c r="K140" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L140" t="str">
         <v>2026-08-19</v>
@@ -7011,7 +7011,7 @@
         <v>LF01043</v>
       </c>
       <c r="K141" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L141" t="str">
         <v>2026-08-19</v>
@@ -7058,7 +7058,7 @@
         <v>LF01043</v>
       </c>
       <c r="K142" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L142" t="str">
         <v>2026-08-19</v>
@@ -7105,7 +7105,7 @@
         <v>LF01043</v>
       </c>
       <c r="K143" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L143" t="str">
         <v>2026-08-19</v>
@@ -7152,7 +7152,7 @@
         <v>LF01043</v>
       </c>
       <c r="K144" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L144" t="str">
         <v>2026-08-19</v>
@@ -7199,7 +7199,7 @@
         <v>LF01043</v>
       </c>
       <c r="K145" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L145" t="str">
         <v>2026-08-19</v>
@@ -7246,7 +7246,7 @@
         <v>LF01043</v>
       </c>
       <c r="K146" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L146" t="str">
         <v>2026-08-19</v>
@@ -7293,7 +7293,7 @@
         <v>LF01043</v>
       </c>
       <c r="K147" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L147" t="str">
         <v>2026-08-19</v>
@@ -7340,7 +7340,7 @@
         <v>LF01043</v>
       </c>
       <c r="K148" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L148" t="str">
         <v>2026-08-19</v>
@@ -7387,7 +7387,7 @@
         <v>LF01043</v>
       </c>
       <c r="K149" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L149" t="str">
         <v>2026-08-19</v>
@@ -7434,7 +7434,7 @@
         <v>LF01043</v>
       </c>
       <c r="K150" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L150" t="str">
         <v>2026-08-19</v>
@@ -7481,7 +7481,7 @@
         <v>LF01043</v>
       </c>
       <c r="K151" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L151" t="str">
         <v>2026-08-19</v>
@@ -7528,7 +7528,7 @@
         <v>LF01043</v>
       </c>
       <c r="K152" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L152" t="str">
         <v>2026-08-19</v>
@@ -7575,7 +7575,7 @@
         <v>LF01043</v>
       </c>
       <c r="K153" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L153" t="str">
         <v>2026-08-19</v>
@@ -7622,7 +7622,7 @@
         <v>LF01043</v>
       </c>
       <c r="K154" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L154" t="str">
         <v>2026-08-19</v>
@@ -7669,7 +7669,7 @@
         <v>LF01043</v>
       </c>
       <c r="K155" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L155" t="str">
         <v>2026-08-19</v>
@@ -7716,7 +7716,7 @@
         <v>LF01043</v>
       </c>
       <c r="K156" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L156" t="str">
         <v>2026-08-19</v>
@@ -7763,7 +7763,7 @@
         <v>LF01043</v>
       </c>
       <c r="K157" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L157" t="str">
         <v>2026-08-19</v>
@@ -7810,7 +7810,7 @@
         <v>LF01043</v>
       </c>
       <c r="K158" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L158" t="str">
         <v>2026-08-19</v>
@@ -7857,7 +7857,7 @@
         <v>iPad (Alex AI)</v>
       </c>
       <c r="K159" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L159" t="str">
         <v>2026-08-19</v>
@@ -7904,7 +7904,7 @@
         <v>iPad (Alex AI)</v>
       </c>
       <c r="K160" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L160" t="str">
         <v>2026-08-19</v>
@@ -7951,7 +7951,7 @@
         <v>AD-Tablet 10"</v>
       </c>
       <c r="K161" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L161" t="str">
         <v>2026-08-19</v>
@@ -7998,7 +7998,7 @@
         <v>AD-Tablet 10"</v>
       </c>
       <c r="K162" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L162" t="str">
         <v>2026-08-19</v>
@@ -8045,7 +8045,7 @@
         <v>AD-Tablet 10"</v>
       </c>
       <c r="K163" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L163" t="str">
         <v>2026-08-19</v>
@@ -8092,7 +8092,7 @@
         <v>UPS 1200W</v>
       </c>
       <c r="K164" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L164" t="str">
         <v>2026-08-19</v>
@@ -8139,7 +8139,7 @@
         <v>UPS 1200W</v>
       </c>
       <c r="K165" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L165" t="str">
         <v>2026-08-19</v>
@@ -8186,7 +8186,7 @@
         <v>IM-PT-PERI</v>
       </c>
       <c r="K166" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L166" t="str">
         <v>2026-08-19</v>
@@ -8233,7 +8233,7 @@
         <v>IM-PT-PERI</v>
       </c>
       <c r="K167" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L167" t="str">
         <v>2026-08-19</v>
@@ -8280,7 +8280,7 @@
         <v>IM-PT-PERI</v>
       </c>
       <c r="K168" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L168" t="str">
         <v>2026-08-19</v>
@@ -8327,7 +8327,7 @@
         <v>Lab Furniture Standard</v>
       </c>
       <c r="K169" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L169" t="str">
         <v>2025-08-01</v>
@@ -8374,7 +8374,7 @@
         <v>Lab Furniture Standard</v>
       </c>
       <c r="K170" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L170" t="str">
         <v>2025-08-01</v>
@@ -8421,7 +8421,7 @@
         <v>Lab Furniture Standard</v>
       </c>
       <c r="K171" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L171" t="str">
         <v>2025-08-01</v>
@@ -8468,7 +8468,7 @@
         <v>Lab Furniture Standard</v>
       </c>
       <c r="K172" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L172" t="str">
         <v>2025-08-01</v>
@@ -8515,7 +8515,7 @@
         <v>Lab Furniture Standard</v>
       </c>
       <c r="K173" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L173" t="str">
         <v>2025-08-01</v>
@@ -8562,7 +8562,7 @@
         <v>Lab Furniture Standard</v>
       </c>
       <c r="K174" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L174" t="str">
         <v>2025-08-01</v>
@@ -8609,7 +8609,7 @@
         <v>Lab Furniture Standard</v>
       </c>
       <c r="K175" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L175" t="str">
         <v>2025-08-01</v>
@@ -8656,7 +8656,7 @@
         <v>Lab Furniture Standard</v>
       </c>
       <c r="K176" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L176" t="str">
         <v>2025-08-01</v>
@@ -8703,7 +8703,7 @@
         <v>Lab Furniture Standard</v>
       </c>
       <c r="K177" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L177" t="str">
         <v>2025-08-01</v>
@@ -8750,7 +8750,7 @@
         <v>Lab Furniture Standard</v>
       </c>
       <c r="K178" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L178" t="str">
         <v>2025-08-01</v>
@@ -8797,7 +8797,7 @@
         <v>Lab Furniture Standard</v>
       </c>
       <c r="K179" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L179" t="str">
         <v>2025-08-01</v>
@@ -8844,7 +8844,7 @@
         <v>Lab Furniture Standard</v>
       </c>
       <c r="K180" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L180" t="str">
         <v>2025-08-01</v>
@@ -8891,7 +8891,7 @@
         <v>Lab Furniture Standard</v>
       </c>
       <c r="K181" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L181" t="str">
         <v>2025-08-01</v>
@@ -8938,7 +8938,7 @@
         <v>Lab Furniture Standard</v>
       </c>
       <c r="K182" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L182" t="str">
         <v>2025-08-01</v>
@@ -8979,7 +8979,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I183" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J183" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9026,7 +9026,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I184" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J184" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9073,7 +9073,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I185" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J185" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9120,7 +9120,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I186" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J186" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9167,7 +9167,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I187" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J187" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9214,7 +9214,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I188" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J188" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9261,7 +9261,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I189" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J189" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9308,7 +9308,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I190" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J190" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9355,7 +9355,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I191" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J191" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9402,7 +9402,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I192" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J192" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9449,7 +9449,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I193" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J193" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9496,7 +9496,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I194" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J194" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9543,7 +9543,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I195" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J195" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9590,7 +9590,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I196" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J196" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9637,7 +9637,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I197" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J197" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9684,7 +9684,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I198" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J198" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9731,7 +9731,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I199" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J199" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9778,7 +9778,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I200" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J200" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9825,7 +9825,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I201" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J201" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9872,7 +9872,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I202" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J202" t="str">
         <v>ไฟฟ้า 3 ไกร์ ราวสไลด์</v>
@@ -9919,7 +9919,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I203" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J203" t="str">
         <v>ไฟฟ้า 2 ไกร์ ราวสไลด์</v>
@@ -9966,7 +9966,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I204" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J204" t="str">
         <v>รุ่นมาตรฐาน</v>
@@ -10013,7 +10013,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I205" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J205" t="str">
         <v>รุ่นมาตรฐาน</v>
@@ -10530,7 +10530,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I216" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J216" t="str">
         <v>รุ่นมาตรฐาน</v>
@@ -10577,7 +10577,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I217" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J217" t="str">
         <v>รุ่นมาตรฐาน</v>
@@ -10624,7 +10624,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I218" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J218" t="str">
         <v>รุ่นมาตรฐาน</v>
@@ -10671,7 +10671,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I219" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J219" t="str">
         <v>รุ่นมาตรฐาน</v>
@@ -10718,7 +10718,7 @@
         <v>2025-05-01</v>
       </c>
       <c r="I220" t="str">
-        <v>Upright Simulation</v>
+        <v>4DEM</v>
       </c>
       <c r="J220" t="str">
         <v>รุ่นมาตรฐาน</v>
@@ -10818,7 +10818,7 @@
         <v>LF00698 Venipuncture Arm</v>
       </c>
       <c r="K222" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L222" t="str">
         <v>2025-06-28</v>
@@ -10865,7 +10865,7 @@
         <v>LF00698 Venipuncture Arm</v>
       </c>
       <c r="K223" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L223" t="str">
         <v>2025-06-28</v>
@@ -10912,7 +10912,7 @@
         <v>LF00698 Venipuncture Arm</v>
       </c>
       <c r="K224" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L224" t="str">
         <v>2025-06-28</v>
@@ -10959,7 +10959,7 @@
         <v>LF00698 Venipuncture Arm</v>
       </c>
       <c r="K225" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L225" t="str">
         <v>2025-06-28</v>
@@ -12275,7 +12275,7 @@
         <v>Anatomical Model Standard</v>
       </c>
       <c r="K253" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L253" t="str">
         <v>2025-06-28</v>
@@ -12322,7 +12322,7 @@
         <v>Anatomical Model Standard</v>
       </c>
       <c r="K254" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L254" t="str">
         <v>2025-06-28</v>
@@ -12369,7 +12369,7 @@
         <v>Anatomical Model Standard</v>
       </c>
       <c r="K255" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L255" t="str">
         <v>2025-06-28</v>
@@ -12416,7 +12416,7 @@
         <v>Anatomical Model Standard</v>
       </c>
       <c r="K256" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L256" t="str">
         <v>2025-06-28</v>
@@ -12463,7 +12463,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K257" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L257" t="str">
         <v>2025-06-28</v>
@@ -12510,7 +12510,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K258" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L258" t="str">
         <v>2025-06-28</v>
@@ -12557,7 +12557,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K259" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L259" t="str">
         <v>2025-06-28</v>
@@ -12604,7 +12604,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K260" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L260" t="str">
         <v>2025-06-28</v>
@@ -12651,7 +12651,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K261" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L261" t="str">
         <v>2025-06-28</v>
@@ -12698,7 +12698,7 @@
         <v>Nursing Manikin Standard</v>
       </c>
       <c r="K262" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L262" t="str">
         <v>2025-06-28</v>
@@ -12745,7 +12745,7 @@
         <v>หุ่น ครุภัณฑ์และอุปกรณ์ในห้องปฏิบัติการพยาบาลการเรียนรู้แบบเสมือนจริง</v>
       </c>
       <c r="K263" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L263" t="str">
         <v>2025-06-28</v>
@@ -12792,7 +12792,7 @@
         <v>P100 Wound Care</v>
       </c>
       <c r="K264" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L264" t="str">
         <v>2025-06-28</v>
@@ -12839,7 +12839,7 @@
         <v>P100 Wound Care</v>
       </c>
       <c r="K265" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L265" t="str">
         <v>2025-06-28</v>
@@ -12886,7 +12886,7 @@
         <v>Birthing Simulator</v>
       </c>
       <c r="K266" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L266" t="str">
         <v>2025-06-28</v>
@@ -12933,7 +12933,7 @@
         <v>Birthing Simulator</v>
       </c>
       <c r="K267" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L267" t="str">
         <v>2025-06-28</v>
@@ -12980,7 +12980,7 @@
         <v>Birthing Simulator</v>
       </c>
       <c r="K268" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L268" t="str">
         <v>2025-06-28</v>
@@ -13027,7 +13027,7 @@
         <v>Birthing Simulator</v>
       </c>
       <c r="K269" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L269" t="str">
         <v>2025-06-28</v>
@@ -13074,7 +13074,7 @@
         <v>Birthing Simulator</v>
       </c>
       <c r="K270" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L270" t="str">
         <v>2025-06-28</v>
@@ -13121,7 +13121,7 @@
         <v>Obstetric Examination Simulator</v>
       </c>
       <c r="K271" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L271" t="str">
         <v>2025-06-28</v>
@@ -13168,7 +13168,7 @@
         <v>Obstetric Examination Simulator</v>
       </c>
       <c r="K272" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L272" t="str">
         <v>2025-06-28</v>
@@ -13215,7 +13215,7 @@
         <v>Baby Care Simulator</v>
       </c>
       <c r="K273" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L273" t="str">
         <v>2025-06-28</v>
@@ -13262,7 +13262,7 @@
         <v>Baby Care Simulator</v>
       </c>
       <c r="K274" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L274" t="str">
         <v>2025-06-28</v>
@@ -13309,7 +13309,7 @@
         <v>Baby Care Simulator</v>
       </c>
       <c r="K275" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L275" t="str">
         <v>2025-06-28</v>
@@ -13356,7 +13356,7 @@
         <v>Baby Care Simulator</v>
       </c>
       <c r="K276" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L276" t="str">
         <v>2025-06-28</v>
@@ -13403,7 +13403,7 @@
         <v>Baby Care Simulator</v>
       </c>
       <c r="K277" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L277" t="str">
         <v>2025-06-28</v>
@@ -13450,7 +13450,7 @@
         <v>718-8804 SAM</v>
       </c>
       <c r="K278" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L278" t="str">
         <v>2025-06-28</v>
@@ -13497,7 +13497,7 @@
         <v>Home Visit Bag Set</v>
       </c>
       <c r="K279" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L279" t="str">
         <v>2025-06-28</v>
@@ -13544,7 +13544,7 @@
         <v>Home Visit Bag Set</v>
       </c>
       <c r="K280" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L280" t="str">
         <v>2025-06-28</v>
@@ -13591,7 +13591,7 @@
         <v>Home Visit Bag Set</v>
       </c>
       <c r="K281" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L281" t="str">
         <v>2025-06-28</v>
@@ -13638,7 +13638,7 @@
         <v>Hospital Bed Standard</v>
       </c>
       <c r="K282" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L282" t="str">
         <v>2025-06-28</v>
@@ -13685,7 +13685,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K283" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L283" t="str">
         <v>2025-06-28</v>
@@ -13732,7 +13732,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K284" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L284" t="str">
         <v>2025-06-28</v>
@@ -13779,7 +13779,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K285" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L285" t="str">
         <v>2025-06-28</v>
@@ -13826,7 +13826,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K286" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L286" t="str">
         <v>2025-06-28</v>
@@ -13873,7 +13873,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K287" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L287" t="str">
         <v>2025-06-28</v>
@@ -13920,7 +13920,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K288" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L288" t="str">
         <v>2025-06-28</v>
@@ -13967,7 +13967,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K289" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L289" t="str">
         <v>2025-06-28</v>
@@ -14014,7 +14014,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K290" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L290" t="str">
         <v>2025-06-28</v>
@@ -14061,7 +14061,7 @@
         <v>มือหมุน 3 ไกร์</v>
       </c>
       <c r="K291" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L291" t="str">
         <v>2025-06-28</v>
@@ -14108,7 +14108,7 @@
         <v>เตียงทำคลอด 2 ตอนปรับระดับ</v>
       </c>
       <c r="K292" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L292" t="str">
         <v>2025-06-28</v>
@@ -14155,7 +14155,7 @@
         <v>เตียงเด็กอ่อนพร้อมเบาะ</v>
       </c>
       <c r="K293" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L293" t="str">
         <v>2025-06-28</v>
@@ -14202,7 +14202,7 @@
         <v>เตียงเด็กอ่อนพร้อมเบาะ</v>
       </c>
       <c r="K294" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L294" t="str">
         <v>2025-06-28</v>
@@ -14249,7 +14249,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K295" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L295" t="str">
         <v>2025-06-28</v>
@@ -14296,7 +14296,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K296" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L296" t="str">
         <v>2025-06-28</v>
@@ -14343,7 +14343,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K297" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L297" t="str">
         <v>2025-06-28</v>
@@ -14390,7 +14390,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K298" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L298" t="str">
         <v>2025-06-28</v>
@@ -14437,7 +14437,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K299" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L299" t="str">
         <v>2025-06-28</v>
@@ -14484,7 +14484,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K300" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L300" t="str">
         <v>2025-06-28</v>
@@ -14531,7 +14531,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K301" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L301" t="str">
         <v>2025-06-28</v>
@@ -14578,7 +14578,7 @@
         <v>Bedside Cabinet</v>
       </c>
       <c r="K302" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L302" t="str">
         <v>2025-06-28</v>
@@ -14625,7 +14625,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K303" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L303" t="str">
         <v>2025-06-28</v>
@@ -14672,7 +14672,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K304" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L304" t="str">
         <v>2025-06-28</v>
@@ -14719,7 +14719,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K305" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L305" t="str">
         <v>2025-06-28</v>
@@ -14766,7 +14766,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K306" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L306" t="str">
         <v>2025-06-28</v>
@@ -14813,7 +14813,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K307" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L307" t="str">
         <v>2025-06-28</v>
@@ -14860,7 +14860,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K308" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L308" t="str">
         <v>2025-06-28</v>
@@ -14907,7 +14907,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K309" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L309" t="str">
         <v>2025-06-28</v>
@@ -14954,7 +14954,7 @@
         <v>Overbed Table</v>
       </c>
       <c r="K310" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L310" t="str">
         <v>2025-06-28</v>
@@ -15001,7 +15001,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K311" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L311" t="str">
         <v>2025-06-28</v>
@@ -15048,7 +15048,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K312" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L312" t="str">
         <v>2025-06-28</v>
@@ -15095,7 +15095,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K313" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L313" t="str">
         <v>2025-06-28</v>
@@ -15142,7 +15142,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K314" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L314" t="str">
         <v>2025-06-28</v>
@@ -15189,7 +15189,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K315" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L315" t="str">
         <v>2025-06-28</v>
@@ -15236,7 +15236,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K316" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L316" t="str">
         <v>2025-06-28</v>
@@ -15283,7 +15283,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K317" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L317" t="str">
         <v>2025-06-28</v>
@@ -15330,7 +15330,7 @@
         <v>Medical Cart Standard</v>
       </c>
       <c r="K318" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L318" t="str">
         <v>2025-06-28</v>
@@ -15377,7 +15377,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K319" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L319" t="str">
         <v>2025-06-28</v>
@@ -15424,7 +15424,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K320" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L320" t="str">
         <v>2025-06-28</v>
@@ -15471,7 +15471,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K321" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L321" t="str">
         <v>2025-06-28</v>
@@ -15518,7 +15518,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K322" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L322" t="str">
         <v>2025-06-28</v>
@@ -15565,7 +15565,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K323" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L323" t="str">
         <v>2025-06-28</v>
@@ -15612,7 +15612,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K324" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L324" t="str">
         <v>2025-06-28</v>
@@ -15659,7 +15659,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K325" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L325" t="str">
         <v>2025-06-28</v>
@@ -15706,7 +15706,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K326" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L326" t="str">
         <v>2025-06-28</v>
@@ -15753,7 +15753,7 @@
         <v>Stainless Waste Bin</v>
       </c>
       <c r="K327" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L327" t="str">
         <v>2025-06-28</v>
@@ -15800,7 +15800,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K328" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L328" t="str">
         <v>2025-06-28</v>
@@ -15847,7 +15847,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K329" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L329" t="str">
         <v>2025-06-28</v>
@@ -15894,7 +15894,7 @@
         <v>Mercurial Sphygmomanometer</v>
       </c>
       <c r="K330" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L330" t="str">
         <v>2025-06-28</v>
@@ -15941,7 +15941,7 @@
         <v>Mercurial Sphygmomanometer</v>
       </c>
       <c r="K331" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L331" t="str">
         <v>2025-06-28</v>
@@ -15988,7 +15988,7 @@
         <v>Mercurial Sphygmomanometer</v>
       </c>
       <c r="K332" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L332" t="str">
         <v>2025-06-28</v>
@@ -16035,7 +16035,7 @@
         <v>Mercurial Sphygmomanometer</v>
       </c>
       <c r="K333" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L333" t="str">
         <v>2025-06-28</v>
@@ -16082,7 +16082,7 @@
         <v>Mercurial Sphygmomanometer</v>
       </c>
       <c r="K334" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L334" t="str">
         <v>2025-06-28</v>
@@ -16129,7 +16129,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K335" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L335" t="str">
         <v>2025-06-28</v>
@@ -16176,7 +16176,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K336" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L336" t="str">
         <v>2025-06-28</v>
@@ -16223,7 +16223,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K337" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L337" t="str">
         <v>2025-06-28</v>
@@ -16270,7 +16270,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K338" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L338" t="str">
         <v>2025-06-28</v>
@@ -16317,7 +16317,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K339" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L339" t="str">
         <v>2025-06-28</v>
@@ -16364,7 +16364,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K340" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L340" t="str">
         <v>2025-06-28</v>
@@ -16411,7 +16411,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K341" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L341" t="str">
         <v>2025-06-28</v>
@@ -16458,7 +16458,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K342" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L342" t="str">
         <v>2025-06-28</v>
@@ -16505,7 +16505,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K343" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L343" t="str">
         <v>2025-06-28</v>
@@ -16552,7 +16552,7 @@
         <v>Digital BP Monitor</v>
       </c>
       <c r="K344" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L344" t="str">
         <v>2025-06-28</v>
@@ -16599,7 +16599,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K345" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L345" t="str">
         <v>2025-06-28</v>
@@ -16646,7 +16646,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K346" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L346" t="str">
         <v>2025-06-28</v>
@@ -16693,7 +16693,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K347" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L347" t="str">
         <v>2025-06-28</v>
@@ -16740,7 +16740,7 @@
         <v>DT-Otoscope</v>
       </c>
       <c r="K348" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L348" t="str">
         <v>2025-06-28</v>
@@ -16787,7 +16787,7 @@
         <v>DT-Ophthalmoscope</v>
       </c>
       <c r="K349" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L349" t="str">
         <v>2025-06-28</v>
@@ -16834,7 +16834,7 @@
         <v>Laryngoscope Set</v>
       </c>
       <c r="K350" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L350" t="str">
         <v>2025-06-28</v>
@@ -16881,7 +16881,7 @@
         <v>Patient Transfer Slide</v>
       </c>
       <c r="K351" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L351" t="str">
         <v>2025-06-28</v>
@@ -16928,7 +16928,7 @@
         <v>Patient Transfer Slide</v>
       </c>
       <c r="K352" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L352" t="str">
         <v>2025-06-28</v>
@@ -16975,7 +16975,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K353" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L353" t="str">
         <v>2025-06-28</v>
@@ -17022,7 +17022,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K354" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L354" t="str">
         <v>2025-06-28</v>
@@ -17069,7 +17069,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K355" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L355" t="str">
         <v>2025-06-28</v>
@@ -17116,7 +17116,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K356" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L356" t="str">
         <v>2025-06-28</v>
@@ -17163,7 +17163,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K357" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L357" t="str">
         <v>2025-06-28</v>
@@ -17210,7 +17210,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K358" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L358" t="str">
         <v>2025-06-28</v>
@@ -17257,7 +17257,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K359" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L359" t="str">
         <v>2025-06-28</v>
@@ -17304,7 +17304,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K360" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L360" t="str">
         <v>2025-06-28</v>
@@ -17351,7 +17351,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K361" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L361" t="str">
         <v>2025-06-28</v>
@@ -17398,7 +17398,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K362" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L362" t="str">
         <v>2025-06-28</v>
@@ -17445,7 +17445,7 @@
         <v>Massage Chair</v>
       </c>
       <c r="K363" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L363" t="str">
         <v>2025-06-28</v>
@@ -17492,7 +17492,7 @@
         <v>Massage Chair</v>
       </c>
       <c r="K364" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L364" t="str">
         <v>2025-06-28</v>
@@ -17539,7 +17539,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K365" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L365" t="str">
         <v>2025-06-28</v>
@@ -17586,7 +17586,7 @@
         <v>Medical Device Standard</v>
       </c>
       <c r="K366" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
       </c>
       <c r="L366" t="str">
         <v>2025-06-28</v>
@@ -17633,7 +17633,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K367" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L367" t="str">
         <v>2025-06-28</v>
@@ -17680,7 +17680,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K368" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L368" t="str">
         <v>2025-06-28</v>
@@ -17727,7 +17727,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K369" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L369" t="str">
         <v>2025-06-28</v>
@@ -17774,7 +17774,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K370" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L370" t="str">
         <v>2025-06-28</v>
@@ -17821,7 +17821,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K371" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L371" t="str">
         <v>2025-06-28</v>
@@ -17868,7 +17868,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K372" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L372" t="str">
         <v>2025-06-28</v>
@@ -17915,7 +17915,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K373" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L373" t="str">
         <v>2025-06-28</v>
@@ -17962,7 +17962,7 @@
         <v>IV Stand Stainless</v>
       </c>
       <c r="K374" t="str">
-        <v>บริษัท อัพไรท์ ซิมมูเลชั่น จำกัด</v>
+        <v/>
       </c>
       <c r="L374" t="str">
         <v>2025-06-28</v>

</xml_diff>

<commit_message>
fix(equipment): update brand for diagnostic sets to Riester (10 items) and digital BP monitors to Omron (10 items)
</commit_message>
<xml_diff>
--- a/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
+++ b/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
@@ -1177,7 +1177,7 @@
         <v>2025-08-19</v>
       </c>
       <c r="I17" t="str">
-        <v>Upright Simulation</v>
+        <v>Riester</v>
       </c>
       <c r="J17" t="str">
         <v>DT-R2050</v>
@@ -1224,7 +1224,7 @@
         <v>2025-08-19</v>
       </c>
       <c r="I18" t="str">
-        <v>Upright Simulation</v>
+        <v>Riester</v>
       </c>
       <c r="J18" t="str">
         <v>DT-R2050</v>
@@ -1271,7 +1271,7 @@
         <v>2025-08-19</v>
       </c>
       <c r="I19" t="str">
-        <v>Upright Simulation</v>
+        <v>Riester</v>
       </c>
       <c r="J19" t="str">
         <v>DT-R2050</v>
@@ -1318,7 +1318,7 @@
         <v>2025-08-19</v>
       </c>
       <c r="I20" t="str">
-        <v>Upright Simulation</v>
+        <v>Riester</v>
       </c>
       <c r="J20" t="str">
         <v>DT-R2050</v>
@@ -1365,7 +1365,7 @@
         <v>2025-08-19</v>
       </c>
       <c r="I21" t="str">
-        <v>Upright Simulation</v>
+        <v>Riester</v>
       </c>
       <c r="J21" t="str">
         <v>DT-R2050</v>
@@ -1412,7 +1412,7 @@
         <v>2025-08-19</v>
       </c>
       <c r="I22" t="str">
-        <v>Upright Simulation</v>
+        <v>Riester</v>
       </c>
       <c r="J22" t="str">
         <v>DT-R2050</v>
@@ -1459,7 +1459,7 @@
         <v>2025-08-19</v>
       </c>
       <c r="I23" t="str">
-        <v>Upright Simulation</v>
+        <v>Riester</v>
       </c>
       <c r="J23" t="str">
         <v>DT-R2050</v>
@@ -1506,7 +1506,7 @@
         <v>2025-08-19</v>
       </c>
       <c r="I24" t="str">
-        <v>Upright Simulation</v>
+        <v>Riester</v>
       </c>
       <c r="J24" t="str">
         <v>DT-R2050</v>
@@ -1553,7 +1553,7 @@
         <v>2025-08-19</v>
       </c>
       <c r="I25" t="str">
-        <v>Upright Simulation</v>
+        <v>Riester</v>
       </c>
       <c r="J25" t="str">
         <v>DT-R2050</v>
@@ -1600,7 +1600,7 @@
         <v>2025-08-19</v>
       </c>
       <c r="I26" t="str">
-        <v>Upright Simulation</v>
+        <v>Riester</v>
       </c>
       <c r="J26" t="str">
         <v>DT-R2050</v>
@@ -16123,7 +16123,7 @@
         <v>2024-06-28</v>
       </c>
       <c r="I335" t="str">
-        <v>Upright Simulation</v>
+        <v>Omron</v>
       </c>
       <c r="J335" t="str">
         <v>Digital BP Monitor</v>
@@ -16170,7 +16170,7 @@
         <v>2024-06-28</v>
       </c>
       <c r="I336" t="str">
-        <v>Upright Simulation</v>
+        <v>Omron</v>
       </c>
       <c r="J336" t="str">
         <v>Digital BP Monitor</v>
@@ -16217,7 +16217,7 @@
         <v>2024-06-28</v>
       </c>
       <c r="I337" t="str">
-        <v>Upright Simulation</v>
+        <v>Omron</v>
       </c>
       <c r="J337" t="str">
         <v>Digital BP Monitor</v>
@@ -16264,7 +16264,7 @@
         <v>2024-06-28</v>
       </c>
       <c r="I338" t="str">
-        <v>Upright Simulation</v>
+        <v>Omron</v>
       </c>
       <c r="J338" t="str">
         <v>Digital BP Monitor</v>
@@ -16311,7 +16311,7 @@
         <v>2024-06-28</v>
       </c>
       <c r="I339" t="str">
-        <v>Upright Simulation</v>
+        <v>Omron</v>
       </c>
       <c r="J339" t="str">
         <v>Digital BP Monitor</v>
@@ -16358,7 +16358,7 @@
         <v>2024-06-28</v>
       </c>
       <c r="I340" t="str">
-        <v>Upright Simulation</v>
+        <v>Omron</v>
       </c>
       <c r="J340" t="str">
         <v>Digital BP Monitor</v>
@@ -16405,7 +16405,7 @@
         <v>2024-06-28</v>
       </c>
       <c r="I341" t="str">
-        <v>Upright Simulation</v>
+        <v>Omron</v>
       </c>
       <c r="J341" t="str">
         <v>Digital BP Monitor</v>
@@ -16452,7 +16452,7 @@
         <v>2024-06-28</v>
       </c>
       <c r="I342" t="str">
-        <v>Upright Simulation</v>
+        <v>Omron</v>
       </c>
       <c r="J342" t="str">
         <v>Digital BP Monitor</v>
@@ -16499,7 +16499,7 @@
         <v>2024-06-28</v>
       </c>
       <c r="I343" t="str">
-        <v>Upright Simulation</v>
+        <v>Omron</v>
       </c>
       <c r="J343" t="str">
         <v>Digital BP Monitor</v>
@@ -16546,7 +16546,7 @@
         <v>2024-06-28</v>
       </c>
       <c r="I344" t="str">
-        <v>Upright Simulation</v>
+        <v>Omron</v>
       </c>
       <c r="J344" t="str">
         <v>Digital BP Monitor</v>

</xml_diff>

<commit_message>
fix(equipment): update image URLs for 8 items (37 assets) from Google Drive links
</commit_message>
<xml_diff>
--- a/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
+++ b/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O374"/>
+  <dimension ref="A1:Q374"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -445,6 +445,12 @@
       <c r="O1" t="str">
         <v>เลขครุภัณฑ์ราชการ</v>
       </c>
+      <c r="P1" t="str">
+        <v>ลิงก์รูปภาพ (Image URL)</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>รูปภาพ</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -2325,6 +2331,12 @@
       <c r="O41" t="str">
         <v>1-B9701-FT17-65450010003/001-68</v>
       </c>
+      <c r="P41" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
+      <c r="Q41" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="str">
@@ -2372,6 +2384,12 @@
       <c r="O42" t="str">
         <v>1-B9701-FT17-65450010003/002-68</v>
       </c>
+      <c r="P42" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
+      <c r="Q42" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="str">
@@ -2419,6 +2437,12 @@
       <c r="O43" t="str">
         <v>1-B9701-FT17-65450010003/003-68</v>
       </c>
+      <c r="P43" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
+      <c r="Q43" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="str">
@@ -2466,6 +2490,12 @@
       <c r="O44" t="str">
         <v>1-B9701-FT17-65450010003/004-68</v>
       </c>
+      <c r="P44" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
+      <c r="Q44" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="str">
@@ -2513,6 +2543,12 @@
       <c r="O45" t="str">
         <v>1-B9701-FT17-65450010003/005-68</v>
       </c>
+      <c r="P45" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
+      <c r="Q45" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="str">
@@ -5192,6 +5228,12 @@
       <c r="O102" t="str">
         <v>1-B9701-FA17-65450010004/045-68</v>
       </c>
+      <c r="P102" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
+      <c r="Q102" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="str">
@@ -5239,6 +5281,12 @@
       <c r="O103" t="str">
         <v>1-B9701-FA17-65450010004/046-68</v>
       </c>
+      <c r="P103" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
+      <c r="Q103" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="str">
@@ -5286,6 +5334,12 @@
       <c r="O104" t="str">
         <v>1-B9701-FA17-65450010004/047-68</v>
       </c>
+      <c r="P104" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
+      <c r="Q104" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="str">
@@ -5333,6 +5387,12 @@
       <c r="O105" t="str">
         <v>1-B9701-FA17-65450010004/048-68</v>
       </c>
+      <c r="P105" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
+      <c r="Q105" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="str">
@@ -5380,6 +5440,12 @@
       <c r="O106" t="str">
         <v>1-B9701-FA17-65450010004/049-68</v>
       </c>
+      <c r="P106" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
+      <c r="Q106" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="str">
@@ -5427,6 +5493,12 @@
       <c r="O107" t="str">
         <v>1-B9701-FA17-65450010004/050-68</v>
       </c>
+      <c r="P107" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
+      <c r="Q107" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="str">
@@ -5474,6 +5546,12 @@
       <c r="O108" t="str">
         <v>1-B9701-FA17-65450010004/051-68</v>
       </c>
+      <c r="P108" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
+      <c r="Q108" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="str">
@@ -5521,6 +5599,12 @@
       <c r="O109" t="str">
         <v>1-B9701-FA17-65450010004/052-68</v>
       </c>
+      <c r="P109" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
+      <c r="Q109" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="str">
@@ -5568,6 +5652,12 @@
       <c r="O110" t="str">
         <v>1-B9701-FA17-65450010004/053-68</v>
       </c>
+      <c r="P110" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
+      <c r="Q110" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
@@ -5615,6 +5705,12 @@
       <c r="O111" t="str">
         <v>1-B9701-FA17-65450010004/054-68</v>
       </c>
+      <c r="P111" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
+      <c r="Q111" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="str">
@@ -9986,6 +10082,12 @@
       <c r="O204" t="str">
         <v>1-B9701-FT17-65450010002/001-68</v>
       </c>
+      <c r="P204" t="str">
+        <v>https://drive.google.com/file/d/1DWZW08_PLRwGlqQl4BoUlhh71GbyPON2/view?usp=sharing</v>
+      </c>
+      <c r="Q204" t="str">
+        <v>https://drive.google.com/file/d/1DWZW08_PLRwGlqQl4BoUlhh71GbyPON2/view?usp=sharing</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="str">
@@ -10080,6 +10182,12 @@
       <c r="O206" t="str">
         <v>1-B9701-FT17-65450010004/001-68</v>
       </c>
+      <c r="P206" t="str">
+        <v>https://drive.google.com/file/d/1KMDffuqSb8cDJ424qT4DNEhzM1LmaWw8/view?usp=drive_link</v>
+      </c>
+      <c r="Q206" t="str">
+        <v>https://drive.google.com/file/d/1KMDffuqSb8cDJ424qT4DNEhzM1LmaWw8/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" t="str">
@@ -10127,6 +10235,12 @@
       <c r="O207" t="str">
         <v>1-B9701-FT17-65450010004/002-68</v>
       </c>
+      <c r="P207" t="str">
+        <v>https://drive.google.com/file/d/1KMDffuqSb8cDJ424qT4DNEhzM1LmaWw8/view?usp=drive_link</v>
+      </c>
+      <c r="Q207" t="str">
+        <v>https://drive.google.com/file/d/1KMDffuqSb8cDJ424qT4DNEhzM1LmaWw8/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="str">
@@ -10174,6 +10288,12 @@
       <c r="O208" t="str">
         <v>1-B9701-FT17-65450010004/003-68</v>
       </c>
+      <c r="P208" t="str">
+        <v>https://drive.google.com/file/d/1KMDffuqSb8cDJ424qT4DNEhzM1LmaWw8/view?usp=drive_link</v>
+      </c>
+      <c r="Q208" t="str">
+        <v>https://drive.google.com/file/d/1KMDffuqSb8cDJ424qT4DNEhzM1LmaWw8/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" t="str">
@@ -10221,6 +10341,12 @@
       <c r="O209" t="str">
         <v>1-B9701-FT17-65450010004/004-68</v>
       </c>
+      <c r="P209" t="str">
+        <v>https://drive.google.com/file/d/1KMDffuqSb8cDJ424qT4DNEhzM1LmaWw8/view?usp=drive_link</v>
+      </c>
+      <c r="Q209" t="str">
+        <v>https://drive.google.com/file/d/1KMDffuqSb8cDJ424qT4DNEhzM1LmaWw8/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="str">
@@ -10268,6 +10394,12 @@
       <c r="O210" t="str">
         <v>1-B9701-FT17-65450010004/005-68</v>
       </c>
+      <c r="P210" t="str">
+        <v>https://drive.google.com/file/d/1KMDffuqSb8cDJ424qT4DNEhzM1LmaWw8/view?usp=drive_link</v>
+      </c>
+      <c r="Q210" t="str">
+        <v>https://drive.google.com/file/d/1KMDffuqSb8cDJ424qT4DNEhzM1LmaWw8/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="str">
@@ -10315,6 +10447,12 @@
       <c r="O211" t="str">
         <v>1-B9701-FT17-65450010004/006-68</v>
       </c>
+      <c r="P211" t="str">
+        <v>https://drive.google.com/file/d/1xyCtKRsHoSu51SrvV2dwPtellv1vdJQK/view?usp=drive_link</v>
+      </c>
+      <c r="Q211" t="str">
+        <v>https://drive.google.com/file/d/1xyCtKRsHoSu51SrvV2dwPtellv1vdJQK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="str">
@@ -10362,6 +10500,12 @@
       <c r="O212" t="str">
         <v>1-B9701-FT17-65450010004/007-68</v>
       </c>
+      <c r="P212" t="str">
+        <v>https://drive.google.com/file/d/1xyCtKRsHoSu51SrvV2dwPtellv1vdJQK/view?usp=drive_link</v>
+      </c>
+      <c r="Q212" t="str">
+        <v>https://drive.google.com/file/d/1xyCtKRsHoSu51SrvV2dwPtellv1vdJQK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="str">
@@ -10409,6 +10553,12 @@
       <c r="O213" t="str">
         <v>1-B9701-FT17-65450010004/008-68</v>
       </c>
+      <c r="P213" t="str">
+        <v>https://drive.google.com/file/d/1xyCtKRsHoSu51SrvV2dwPtellv1vdJQK/view?usp=drive_link</v>
+      </c>
+      <c r="Q213" t="str">
+        <v>https://drive.google.com/file/d/1xyCtKRsHoSu51SrvV2dwPtellv1vdJQK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="str">
@@ -10456,6 +10606,12 @@
       <c r="O214" t="str">
         <v>1-B9701-FT17-65450010004/009-68</v>
       </c>
+      <c r="P214" t="str">
+        <v>https://drive.google.com/file/d/1xyCtKRsHoSu51SrvV2dwPtellv1vdJQK/view?usp=drive_link</v>
+      </c>
+      <c r="Q214" t="str">
+        <v>https://drive.google.com/file/d/1xyCtKRsHoSu51SrvV2dwPtellv1vdJQK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="str">
@@ -10503,6 +10659,12 @@
       <c r="O215" t="str">
         <v>1-B9701-FT17-65450010004/010-68</v>
       </c>
+      <c r="P215" t="str">
+        <v>https://drive.google.com/file/d/1xyCtKRsHoSu51SrvV2dwPtellv1vdJQK/view?usp=drive_link</v>
+      </c>
+      <c r="Q215" t="str">
+        <v>https://drive.google.com/file/d/1xyCtKRsHoSu51SrvV2dwPtellv1vdJQK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="str">
@@ -10785,6 +10947,12 @@
       <c r="O221" t="str">
         <v>1-B9701-FT17-65450010004/016-68</v>
       </c>
+      <c r="P221" t="str">
+        <v>https://drive.google.com/file/d/1kiOynTyquGIhurpptqoCWFk2f4YJTzt-/view?usp=sharing</v>
+      </c>
+      <c r="Q221" t="str">
+        <v>https://drive.google.com/file/d/1kiOynTyquGIhurpptqoCWFk2f4YJTzt-/view?usp=sharing</v>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="str">
@@ -11819,6 +11987,12 @@
       <c r="O243" t="str">
         <v>1-B9701-FT17-65450010004/034-68</v>
       </c>
+      <c r="P243" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
+      <c r="Q243" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="244">
       <c r="A244" t="str">
@@ -11866,6 +12040,12 @@
       <c r="O244" t="str">
         <v>1-B9701-FT17-65450010004/035-68</v>
       </c>
+      <c r="P244" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
+      <c r="Q244" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="245">
       <c r="A245" t="str">
@@ -11913,6 +12093,12 @@
       <c r="O245" t="str">
         <v>1-B9701-FT17-65450010004/036-68</v>
       </c>
+      <c r="P245" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
+      <c r="Q245" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="246">
       <c r="A246" t="str">
@@ -11960,6 +12146,12 @@
       <c r="O246" t="str">
         <v>1-B9701-FT17-65450010004/037-68</v>
       </c>
+      <c r="P246" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
+      <c r="Q246" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="247">
       <c r="A247" t="str">
@@ -12007,6 +12199,12 @@
       <c r="O247" t="str">
         <v>1-B9701-FT17-65450010004/038-68</v>
       </c>
+      <c r="P247" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
+      <c r="Q247" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="248">
       <c r="A248" t="str">
@@ -12054,6 +12252,12 @@
       <c r="O248" t="str">
         <v>1-B9701-FT17-65450010004/039-68</v>
       </c>
+      <c r="P248" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
+      <c r="Q248" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="249">
       <c r="A249" t="str">
@@ -12101,6 +12305,12 @@
       <c r="O249" t="str">
         <v>1-B9701-FT17-65450010004/040-68</v>
       </c>
+      <c r="P249" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
+      <c r="Q249" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="250">
       <c r="A250" t="str">
@@ -12148,6 +12358,12 @@
       <c r="O250" t="str">
         <v>1-B9701-FT17-65450010004/041-68</v>
       </c>
+      <c r="P250" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
+      <c r="Q250" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="251">
       <c r="A251" t="str">
@@ -12195,6 +12411,12 @@
       <c r="O251" t="str">
         <v>1-B9701-FT17-65450010004/042-68</v>
       </c>
+      <c r="P251" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
+      <c r="Q251" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="252">
       <c r="A252" t="str">
@@ -12242,6 +12464,12 @@
       <c r="O252" t="str">
         <v>1-B9701-FT17-65450010004/043-68</v>
       </c>
+      <c r="P252" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
+      <c r="Q252" t="str">
+        <v>https://drive.google.com/file/d/1I3j4FtFdzZNOq74M-lt01NwuHRQca8va/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="253">
       <c r="A253" t="str">
@@ -17979,7 +18207,7 @@
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O374"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q374"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(equipment): update images for 13 items (44 assets) from filled Excel report
</commit_message>
<xml_diff>
--- a/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
+++ b/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
@@ -1767,6 +1767,12 @@
       <c r="O29" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (46-1/2)</v>
       </c>
+      <c r="P29" t="str">
+        <v>https://drive.google.com/file/d/1WwxEXRR9BQt6Mew5Ag7c2pe9aGR41mhL/view?usp=sharing</v>
+      </c>
+      <c r="Q29" t="str">
+        <v>https://drive.google.com/file/d/1WwxEXRR9BQt6Mew5Ag7c2pe9aGR41mhL/view?usp=sharing</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1814,6 +1820,12 @@
       <c r="O30" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (46-2/2)</v>
       </c>
+      <c r="P30" t="str">
+        <v>https://drive.google.com/file/d/1WwxEXRR9BQt6Mew5Ag7c2pe9aGR41mhL/view?usp=sharing</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>https://drive.google.com/file/d/1WwxEXRR9BQt6Mew5Ag7c2pe9aGR41mhL/view?usp=sharing</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1861,6 +1873,12 @@
       <c r="O31" t="str">
         <v>1-B9701-FA17-65150840001/003-68</v>
       </c>
+      <c r="P31" t="str">
+        <v>https://drive.google.com/file/d/1WwxEXRR9BQt6Mew5Ag7c2pe9aGR41mhL/view?usp=sharing</v>
+      </c>
+      <c r="Q31" t="str">
+        <v>https://drive.google.com/file/d/1WwxEXRR9BQt6Mew5Ag7c2pe9aGR41mhL/view?usp=sharing</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
@@ -1908,6 +1926,12 @@
       <c r="O32" t="str">
         <v>1-B9701-FA17-65150840001/004-68</v>
       </c>
+      <c r="P32" t="str">
+        <v>https://drive.google.com/file/d/1WwxEXRR9BQt6Mew5Ag7c2pe9aGR41mhL/view?usp=sharing</v>
+      </c>
+      <c r="Q32" t="str">
+        <v>https://drive.google.com/file/d/1WwxEXRR9BQt6Mew5Ag7c2pe9aGR41mhL/view?usp=sharing</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
@@ -1955,6 +1979,12 @@
       <c r="O33" t="str">
         <v>1-B9701-FA17-65150840001/005-68</v>
       </c>
+      <c r="P33" t="str">
+        <v>https://drive.google.com/file/d/1WwxEXRR9BQt6Mew5Ag7c2pe9aGR41mhL/view?usp=sharing</v>
+      </c>
+      <c r="Q33" t="str">
+        <v>https://drive.google.com/file/d/1WwxEXRR9BQt6Mew5Ag7c2pe9aGR41mhL/view?usp=sharing</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
@@ -2002,6 +2032,12 @@
       <c r="O34" t="str">
         <v>1-B9701-FA17-65150840001/006-68</v>
       </c>
+      <c r="P34" t="str">
+        <v>https://drive.google.com/file/d/1WwxEXRR9BQt6Mew5Ag7c2pe9aGR41mhL/view?usp=sharing</v>
+      </c>
+      <c r="Q34" t="str">
+        <v>https://drive.google.com/file/d/1WwxEXRR9BQt6Mew5Ag7c2pe9aGR41mhL/view?usp=sharing</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
@@ -2049,6 +2085,12 @@
       <c r="O35" t="str">
         <v>1-B9701-FA17-65150840001/007-68</v>
       </c>
+      <c r="P35" t="str">
+        <v>https://drive.google.com/file/d/1WwxEXRR9BQt6Mew5Ag7c2pe9aGR41mhL/view?usp=sharing</v>
+      </c>
+      <c r="Q35" t="str">
+        <v>https://drive.google.com/file/d/1WwxEXRR9BQt6Mew5Ag7c2pe9aGR41mhL/view?usp=sharing</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
@@ -2237,6 +2279,12 @@
       <c r="O39" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (6-1/2)</v>
       </c>
+      <c r="P39" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
+      <c r="Q39" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="str">
@@ -2284,6 +2332,12 @@
       <c r="O40" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (6-2/2)</v>
       </c>
+      <c r="P40" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
+      <c r="Q40" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="str">
@@ -2596,6 +2650,12 @@
       <c r="O46" t="str">
         <v>1-B9701-FA17-65450010003/001-68</v>
       </c>
+      <c r="P46" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
+      <c r="Q46" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="str">
@@ -2643,6 +2703,12 @@
       <c r="O47" t="str">
         <v>1-B9701-FA17-65450010003/002-68</v>
       </c>
+      <c r="P47" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
+      <c r="Q47" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="str">
@@ -2690,6 +2756,12 @@
       <c r="O48" t="str">
         <v>1-B9701-FA17-65450010003/003-68</v>
       </c>
+      <c r="P48" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
+      <c r="Q48" t="str">
+        <v>https://drive.google.com/file/d/1qWDRLyiRBRWXFeMUaNj08d7du6_Nq4v0/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="str">
@@ -2737,6 +2809,12 @@
       <c r="O49" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (20-1/2)</v>
       </c>
+      <c r="P49" t="str">
+        <v>https://drive.google.com/file/d/1xhCa_pvJQQFP3gynGHmQwdQVFiHDhHHC/view?usp=drive_link</v>
+      </c>
+      <c r="Q49" t="str">
+        <v>https://drive.google.com/file/d/1xhCa_pvJQQFP3gynGHmQwdQVFiHDhHHC/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="str">
@@ -2784,6 +2862,12 @@
       <c r="O50" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (20-2/2)</v>
       </c>
+      <c r="P50" t="str">
+        <v>https://drive.google.com/file/d/1xhCa_pvJQQFP3gynGHmQwdQVFiHDhHHC/view?usp=drive_link</v>
+      </c>
+      <c r="Q50" t="str">
+        <v>https://drive.google.com/file/d/1xhCa_pvJQQFP3gynGHmQwdQVFiHDhHHC/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="str">
@@ -4241,6 +4325,12 @@
       <c r="O81" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (10-1/1)</v>
       </c>
+      <c r="P81" t="str">
+        <v>https://drive.google.com/file/d/1h2zDqKk0b21Y49tWDiH8OIEWSgI0UBJe/view?usp=drive_link</v>
+      </c>
+      <c r="Q81" t="str">
+        <v>https://drive.google.com/file/d/1h2zDqKk0b21Y49tWDiH8OIEWSgI0UBJe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="str">
@@ -4288,6 +4378,12 @@
       <c r="O82" t="str">
         <v>1-B9701-FA17-65450010004/027-68</v>
       </c>
+      <c r="P82" t="str">
+        <v>https://drive.google.com/file/d/1h2zDqKk0b21Y49tWDiH8OIEWSgI0UBJe/view?usp=drive_link</v>
+      </c>
+      <c r="Q82" t="str">
+        <v>https://drive.google.com/file/d/1h2zDqKk0b21Y49tWDiH8OIEWSgI0UBJe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="str">
@@ -4335,6 +4431,12 @@
       <c r="O83" t="str">
         <v>1-B9701-FA17-65450010004/028-68</v>
       </c>
+      <c r="P83" t="str">
+        <v>https://drive.google.com/file/d/1h2zDqKk0b21Y49tWDiH8OIEWSgI0UBJe/view?usp=drive_link</v>
+      </c>
+      <c r="Q83" t="str">
+        <v>https://drive.google.com/file/d/1h2zDqKk0b21Y49tWDiH8OIEWSgI0UBJe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="str">
@@ -4382,6 +4484,12 @@
       <c r="O84" t="str">
         <v>1-B9701-FA17-65450010004/029-68</v>
       </c>
+      <c r="P84" t="str">
+        <v>https://drive.google.com/file/d/1h2zDqKk0b21Y49tWDiH8OIEWSgI0UBJe/view?usp=drive_link</v>
+      </c>
+      <c r="Q84" t="str">
+        <v>https://drive.google.com/file/d/1h2zDqKk0b21Y49tWDiH8OIEWSgI0UBJe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="str">
@@ -4429,6 +4537,12 @@
       <c r="O85" t="str">
         <v>1-B9701-FA17-65450010004/030-68</v>
       </c>
+      <c r="P85" t="str">
+        <v>https://drive.google.com/file/d/1h2zDqKk0b21Y49tWDiH8OIEWSgI0UBJe/view?usp=drive_link</v>
+      </c>
+      <c r="Q85" t="str">
+        <v>https://drive.google.com/file/d/1h2zDqKk0b21Y49tWDiH8OIEWSgI0UBJe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="str">
@@ -4476,6 +4590,12 @@
       <c r="O86" t="str">
         <v>1-B9701-FA17-65450010004/031-68</v>
       </c>
+      <c r="P86" t="str">
+        <v>https://drive.google.com/file/d/1h2zDqKk0b21Y49tWDiH8OIEWSgI0UBJe/view?usp=drive_link</v>
+      </c>
+      <c r="Q86" t="str">
+        <v>https://drive.google.com/file/d/1h2zDqKk0b21Y49tWDiH8OIEWSgI0UBJe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="str">
@@ -5134,6 +5254,12 @@
       <c r="O100" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (13-1/2)</v>
       </c>
+      <c r="P100" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
+      <c r="Q100" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="str">
@@ -5181,6 +5307,12 @@
       <c r="O101" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (13-2/2)</v>
       </c>
+      <c r="P101" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
+      <c r="Q101" t="str">
+        <v>https://drive.google.com/file/d/1BKFWzzaVlnwr6u5W10lyJMxDFtTqV6oX/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="str">
@@ -10712,6 +10844,12 @@
       <c r="O216" t="str">
         <v>1-B9701-FT17-65450010004/011-68</v>
       </c>
+      <c r="P216" t="str">
+        <v>https://drive.google.com/file/d/1pVekl9EOGsZa7r8cAnOLMPKB8HZwUFou/view?usp=drive_link</v>
+      </c>
+      <c r="Q216" t="str">
+        <v>https://drive.google.com/file/d/1pVekl9EOGsZa7r8cAnOLMPKB8HZwUFou/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="str">
@@ -10759,6 +10897,12 @@
       <c r="O217" t="str">
         <v>1-B9701-FT17-65450010004/012-68</v>
       </c>
+      <c r="P217" t="str">
+        <v>https://drive.google.com/file/d/1pVekl9EOGsZa7r8cAnOLMPKB8HZwUFou/view?usp=drive_link</v>
+      </c>
+      <c r="Q217" t="str">
+        <v>https://drive.google.com/file/d/1pVekl9EOGsZa7r8cAnOLMPKB8HZwUFou/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="str">
@@ -10806,6 +10950,12 @@
       <c r="O218" t="str">
         <v>1-B9701-FT17-65450010004/013-68</v>
       </c>
+      <c r="P218" t="str">
+        <v>https://drive.google.com/file/d/1pVekl9EOGsZa7r8cAnOLMPKB8HZwUFou/view?usp=drive_link</v>
+      </c>
+      <c r="Q218" t="str">
+        <v>https://drive.google.com/file/d/1pVekl9EOGsZa7r8cAnOLMPKB8HZwUFou/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="str">
@@ -10853,6 +11003,12 @@
       <c r="O219" t="str">
         <v>1-B9701-FT17-65450010004/014-68</v>
       </c>
+      <c r="P219" t="str">
+        <v>https://drive.google.com/file/d/1pVekl9EOGsZa7r8cAnOLMPKB8HZwUFou/view?usp=drive_link</v>
+      </c>
+      <c r="Q219" t="str">
+        <v>https://drive.google.com/file/d/1pVekl9EOGsZa7r8cAnOLMPKB8HZwUFou/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="str">
@@ -10900,6 +11056,12 @@
       <c r="O220" t="str">
         <v>1-B9701-FT17-65450010004/015-68</v>
       </c>
+      <c r="P220" t="str">
+        <v>https://drive.google.com/file/d/1pVekl9EOGsZa7r8cAnOLMPKB8HZwUFou/view?usp=drive_link</v>
+      </c>
+      <c r="Q220" t="str">
+        <v>https://drive.google.com/file/d/1pVekl9EOGsZa7r8cAnOLMPKB8HZwUFou/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="str">
@@ -11000,6 +11162,12 @@
       <c r="O222" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (11-1/4)</v>
       </c>
+      <c r="P222" t="str">
+        <v>https://drive.google.com/file/d/1Pvgj6-kJvOs9zstAtbjtngUe65sMnbST/view?usp=drive_link</v>
+      </c>
+      <c r="Q222" t="str">
+        <v>https://drive.google.com/file/d/1Pvgj6-kJvOs9zstAtbjtngUe65sMnbST/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="str">
@@ -11047,6 +11215,12 @@
       <c r="O223" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (11-2/4)</v>
       </c>
+      <c r="P223" t="str">
+        <v>https://drive.google.com/file/d/1Pvgj6-kJvOs9zstAtbjtngUe65sMnbST/view?usp=drive_link</v>
+      </c>
+      <c r="Q223" t="str">
+        <v>https://drive.google.com/file/d/1Pvgj6-kJvOs9zstAtbjtngUe65sMnbST/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="224">
       <c r="A224" t="str">
@@ -11094,6 +11268,12 @@
       <c r="O224" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (11-3/4)</v>
       </c>
+      <c r="P224" t="str">
+        <v>https://drive.google.com/file/d/1Pvgj6-kJvOs9zstAtbjtngUe65sMnbST/view?usp=drive_link</v>
+      </c>
+      <c r="Q224" t="str">
+        <v>https://drive.google.com/file/d/1Pvgj6-kJvOs9zstAtbjtngUe65sMnbST/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="str">
@@ -11141,6 +11321,12 @@
       <c r="O225" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (11-4/4)</v>
       </c>
+      <c r="P225" t="str">
+        <v>https://drive.google.com/file/d/1Pvgj6-kJvOs9zstAtbjtngUe65sMnbST/view?usp=drive_link</v>
+      </c>
+      <c r="Q225" t="str">
+        <v>https://drive.google.com/file/d/1Pvgj6-kJvOs9zstAtbjtngUe65sMnbST/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="str">
@@ -11188,6 +11374,12 @@
       <c r="O226" t="str">
         <v>1-B9701-FT17-65450010004/017-68</v>
       </c>
+      <c r="P226" t="str">
+        <v>https://drive.google.com/file/d/1RxesQCI5Qog424F4ONVz6_MpV1EhV-nw/view?usp=drive_link</v>
+      </c>
+      <c r="Q226" t="str">
+        <v>https://drive.google.com/file/d/1RxesQCI5Qog424F4ONVz6_MpV1EhV-nw/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="str">
@@ -11235,6 +11427,12 @@
       <c r="O227" t="str">
         <v>1-B9701-FT17-65450010004/018-68</v>
       </c>
+      <c r="P227" t="str">
+        <v>https://drive.google.com/file/d/1RxesQCI5Qog424F4ONVz6_MpV1EhV-nw/view?usp=drive_link</v>
+      </c>
+      <c r="Q227" t="str">
+        <v>https://drive.google.com/file/d/1RxesQCI5Qog424F4ONVz6_MpV1EhV-nw/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="str">
@@ -11282,6 +11480,12 @@
       <c r="O228" t="str">
         <v>1-B9701-FT17-65450010004/019-68</v>
       </c>
+      <c r="P228" t="str">
+        <v>https://drive.google.com/file/d/1RxesQCI5Qog424F4ONVz6_MpV1EhV-nw/view?usp=drive_link</v>
+      </c>
+      <c r="Q228" t="str">
+        <v>https://drive.google.com/file/d/1RxesQCI5Qog424F4ONVz6_MpV1EhV-nw/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="str">
@@ -11329,6 +11533,12 @@
       <c r="O229" t="str">
         <v>1-B9701-FT17-65450010004/020-68</v>
       </c>
+      <c r="P229" t="str">
+        <v>https://drive.google.com/file/d/1RxesQCI5Qog424F4ONVz6_MpV1EhV-nw/view?usp=drive_link</v>
+      </c>
+      <c r="Q229" t="str">
+        <v>https://drive.google.com/file/d/1RxesQCI5Qog424F4ONVz6_MpV1EhV-nw/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="str">
@@ -11376,6 +11586,12 @@
       <c r="O230" t="str">
         <v>1-B9701-FT17-65450010004/021-68</v>
       </c>
+      <c r="P230" t="str">
+        <v>https://drive.google.com/file/d/1RxesQCI5Qog424F4ONVz6_MpV1EhV-nw/view?usp=drive_link</v>
+      </c>
+      <c r="Q230" t="str">
+        <v>https://drive.google.com/file/d/1RxesQCI5Qog424F4ONVz6_MpV1EhV-nw/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="str">
@@ -11423,6 +11639,12 @@
       <c r="O231" t="str">
         <v>1-B9701-FT17-65450010004/022-68</v>
       </c>
+      <c r="P231" t="str">
+        <v>https://drive.google.com/file/d/1RxesQCI5Qog424F4ONVz6_MpV1EhV-nw/view?usp=drive_link</v>
+      </c>
+      <c r="Q231" t="str">
+        <v>https://drive.google.com/file/d/1RxesQCI5Qog424F4ONVz6_MpV1EhV-nw/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="str">
@@ -11470,6 +11692,12 @@
       <c r="O232" t="str">
         <v>1-B9701-FT17-65450010004/023-68</v>
       </c>
+      <c r="P232" t="str">
+        <v>https://drive.google.com/file/d/1RxesQCI5Qog424F4ONVz6_MpV1EhV-nw/view?usp=drive_link</v>
+      </c>
+      <c r="Q232" t="str">
+        <v>https://drive.google.com/file/d/1RxesQCI5Qog424F4ONVz6_MpV1EhV-nw/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="str">
@@ -11517,6 +11745,12 @@
       <c r="O233" t="str">
         <v>1-B9701-FT17-65450010004/024-68</v>
       </c>
+      <c r="P233" t="str">
+        <v>https://drive.google.com/file/d/1_uxkwQ9se7IoOdrW4w1FPQCmFIgGh2qk/view?usp=drive_link</v>
+      </c>
+      <c r="Q233" t="str">
+        <v>https://drive.google.com/file/d/1_uxkwQ9se7IoOdrW4w1FPQCmFIgGh2qk/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="str">
@@ -11564,6 +11798,12 @@
       <c r="O234" t="str">
         <v>1-B9701-FT17-65450010004/025-68</v>
       </c>
+      <c r="P234" t="str">
+        <v>https://drive.google.com/file/d/1_uxkwQ9se7IoOdrW4w1FPQCmFIgGh2qk/view?usp=drive_link</v>
+      </c>
+      <c r="Q234" t="str">
+        <v>https://drive.google.com/file/d/1_uxkwQ9se7IoOdrW4w1FPQCmFIgGh2qk/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="str">
@@ -11611,6 +11851,12 @@
       <c r="O235" t="str">
         <v>1-B9701-FT17-65450010004/026-68</v>
       </c>
+      <c r="P235" t="str">
+        <v>https://drive.google.com/file/d/1_uxkwQ9se7IoOdrW4w1FPQCmFIgGh2qk/view?usp=drive_link</v>
+      </c>
+      <c r="Q235" t="str">
+        <v>https://drive.google.com/file/d/1_uxkwQ9se7IoOdrW4w1FPQCmFIgGh2qk/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
@@ -11658,6 +11904,12 @@
       <c r="O236" t="str">
         <v>1-B9701-FT17-65450010004/027-68</v>
       </c>
+      <c r="P236" t="str">
+        <v>https://drive.google.com/file/d/1_uxkwQ9se7IoOdrW4w1FPQCmFIgGh2qk/view?usp=drive_link</v>
+      </c>
+      <c r="Q236" t="str">
+        <v>https://drive.google.com/file/d/1_uxkwQ9se7IoOdrW4w1FPQCmFIgGh2qk/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="str">
@@ -11705,6 +11957,12 @@
       <c r="O237" t="str">
         <v>1-B9701-FT17-65450010004/028-68</v>
       </c>
+      <c r="P237" t="str">
+        <v>https://drive.google.com/file/d/1_uxkwQ9se7IoOdrW4w1FPQCmFIgGh2qk/view?usp=drive_link</v>
+      </c>
+      <c r="Q237" t="str">
+        <v>https://drive.google.com/file/d/1_uxkwQ9se7IoOdrW4w1FPQCmFIgGh2qk/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="str">
@@ -11752,6 +12010,12 @@
       <c r="O238" t="str">
         <v>1-B9701-FT17-65450010004/029-68</v>
       </c>
+      <c r="P238" t="str">
+        <v>https://drive.google.com/file/d/1LaQFTimV6MZPolqp5xQKMqzPFS-TaEhv/view?usp=drive_link</v>
+      </c>
+      <c r="Q238" t="str">
+        <v>https://drive.google.com/file/d/1LaQFTimV6MZPolqp5xQKMqzPFS-TaEhv/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="str">
@@ -11799,6 +12063,12 @@
       <c r="O239" t="str">
         <v>1-B9701-FT17-65450010004/030-68</v>
       </c>
+      <c r="P239" t="str">
+        <v>https://drive.google.com/file/d/1LaQFTimV6MZPolqp5xQKMqzPFS-TaEhv/view?usp=drive_link</v>
+      </c>
+      <c r="Q239" t="str">
+        <v>https://drive.google.com/file/d/1LaQFTimV6MZPolqp5xQKMqzPFS-TaEhv/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="240">
       <c r="A240" t="str">
@@ -11846,6 +12116,12 @@
       <c r="O240" t="str">
         <v>1-B9701-FT17-65450010004/031-68</v>
       </c>
+      <c r="P240" t="str">
+        <v>https://drive.google.com/file/d/1LaQFTimV6MZPolqp5xQKMqzPFS-TaEhv/view?usp=drive_link</v>
+      </c>
+      <c r="Q240" t="str">
+        <v>https://drive.google.com/file/d/1LaQFTimV6MZPolqp5xQKMqzPFS-TaEhv/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="241">
       <c r="A241" t="str">
@@ -11893,6 +12169,12 @@
       <c r="O241" t="str">
         <v>1-B9701-FT17-65450010004/032-68</v>
       </c>
+      <c r="P241" t="str">
+        <v>https://drive.google.com/file/d/1LaQFTimV6MZPolqp5xQKMqzPFS-TaEhv/view?usp=drive_link</v>
+      </c>
+      <c r="Q241" t="str">
+        <v>https://drive.google.com/file/d/1LaQFTimV6MZPolqp5xQKMqzPFS-TaEhv/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="242">
       <c r="A242" t="str">
@@ -11940,6 +12222,12 @@
       <c r="O242" t="str">
         <v>1-B9701-FT17-65450010004/033-68</v>
       </c>
+      <c r="P242" t="str">
+        <v>https://drive.google.com/file/d/1LaQFTimV6MZPolqp5xQKMqzPFS-TaEhv/view?usp=drive_link</v>
+      </c>
+      <c r="Q242" t="str">
+        <v>https://drive.google.com/file/d/1LaQFTimV6MZPolqp5xQKMqzPFS-TaEhv/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="243">
       <c r="A243" t="str">
@@ -12517,6 +12805,12 @@
       <c r="O253" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (1-1/1)</v>
       </c>
+      <c r="P253" t="str">
+        <v>https://drive.google.com/file/d/1_A1FFkoUcQAblApAAnHbNz0hXbTArRbN/view?usp=sharing</v>
+      </c>
+      <c r="Q253" t="str">
+        <v>https://drive.google.com/file/d/1_A1FFkoUcQAblApAAnHbNz0hXbTArRbN/view?usp=sharing</v>
+      </c>
     </row>
     <row r="254">
       <c r="A254" t="str">
@@ -12564,6 +12858,12 @@
       <c r="O254" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (2-1/1)</v>
       </c>
+      <c r="P254" t="str">
+        <v>https://drive.google.com/file/d/1Q_KelcnuhLEZZ9erVef-opp_mIrJbgTQ/view?usp=drive_link</v>
+      </c>
+      <c r="Q254" t="str">
+        <v>https://drive.google.com/file/d/1Q_KelcnuhLEZZ9erVef-opp_mIrJbgTQ/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="str">
@@ -12611,6 +12911,12 @@
       <c r="O255" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (3-1/1)</v>
       </c>
+      <c r="P255" t="str">
+        <v>https://drive.google.com/file/d/1dNc97jEKO0NXVuOUnZIfQ7xfRlg9mDP_/view?usp=drive_link</v>
+      </c>
+      <c r="Q255" t="str">
+        <v>https://drive.google.com/file/d/1dNc97jEKO0NXVuOUnZIfQ7xfRlg9mDP_/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="256">
       <c r="A256" t="str">
@@ -12658,6 +12964,12 @@
       <c r="O256" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (4-1/1)</v>
       </c>
+      <c r="P256" t="str">
+        <v>https://drive.google.com/file/d/1UHr2xqmXLbClpRfqEL-rdr-FMsI2Q40Q/view?usp=sharing</v>
+      </c>
+      <c r="Q256" t="str">
+        <v>https://drive.google.com/file/d/1UHr2xqmXLbClpRfqEL-rdr-FMsI2Q40Q/view?usp=sharing</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="str">
@@ -12705,6 +13017,12 @@
       <c r="O257" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (5-1/6)</v>
       </c>
+      <c r="P257" t="str">
+        <v>https://drive.google.com/file/d/1X23FDFYBaumRSFAy8D2iq3B8GkyVqpkA/view?usp=drive_link</v>
+      </c>
+      <c r="Q257" t="str">
+        <v>https://drive.google.com/file/d/1X23FDFYBaumRSFAy8D2iq3B8GkyVqpkA/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" t="str">
@@ -12752,6 +13070,12 @@
       <c r="O258" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (5-2/6)</v>
       </c>
+      <c r="P258" t="str">
+        <v>https://drive.google.com/file/d/1X23FDFYBaumRSFAy8D2iq3B8GkyVqpkA/view?usp=drive_link</v>
+      </c>
+      <c r="Q258" t="str">
+        <v>https://drive.google.com/file/d/1X23FDFYBaumRSFAy8D2iq3B8GkyVqpkA/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="str">
@@ -12799,6 +13123,12 @@
       <c r="O259" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (5-3/6)</v>
       </c>
+      <c r="P259" t="str">
+        <v>https://drive.google.com/file/d/1X23FDFYBaumRSFAy8D2iq3B8GkyVqpkA/view?usp=drive_link</v>
+      </c>
+      <c r="Q259" t="str">
+        <v>https://drive.google.com/file/d/1X23FDFYBaumRSFAy8D2iq3B8GkyVqpkA/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="260">
       <c r="A260" t="str">
@@ -12846,6 +13176,12 @@
       <c r="O260" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (5-4/6)</v>
       </c>
+      <c r="P260" t="str">
+        <v>https://drive.google.com/file/d/1X23FDFYBaumRSFAy8D2iq3B8GkyVqpkA/view?usp=drive_link</v>
+      </c>
+      <c r="Q260" t="str">
+        <v>https://drive.google.com/file/d/1X23FDFYBaumRSFAy8D2iq3B8GkyVqpkA/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="261">
       <c r="A261" t="str">
@@ -12893,6 +13229,12 @@
       <c r="O261" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (5-5/6)</v>
       </c>
+      <c r="P261" t="str">
+        <v>https://drive.google.com/file/d/1X23FDFYBaumRSFAy8D2iq3B8GkyVqpkA/view?usp=drive_link</v>
+      </c>
+      <c r="Q261" t="str">
+        <v>https://drive.google.com/file/d/1X23FDFYBaumRSFAy8D2iq3B8GkyVqpkA/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="262">
       <c r="A262" t="str">
@@ -12940,6 +13282,12 @@
       <c r="O262" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (5-6/6)</v>
       </c>
+      <c r="P262" t="str">
+        <v>https://drive.google.com/file/d/1X23FDFYBaumRSFAy8D2iq3B8GkyVqpkA/view?usp=drive_link</v>
+      </c>
+      <c r="Q262" t="str">
+        <v>https://drive.google.com/file/d/1X23FDFYBaumRSFAy8D2iq3B8GkyVqpkA/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="263">
       <c r="A263" t="str">
@@ -13128,6 +13476,12 @@
       <c r="O266" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (14-1/5)</v>
       </c>
+      <c r="P266" t="str">
+        <v>https://drive.google.com/file/d/1gUIW3ZmoWKt8lb7-YLmh3cXe2c8XkO6o/view?usp=drive_link</v>
+      </c>
+      <c r="Q266" t="str">
+        <v>https://drive.google.com/file/d/1gUIW3ZmoWKt8lb7-YLmh3cXe2c8XkO6o/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="267">
       <c r="A267" t="str">
@@ -13175,6 +13529,12 @@
       <c r="O267" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (14-2/5)</v>
       </c>
+      <c r="P267" t="str">
+        <v>https://drive.google.com/file/d/1gUIW3ZmoWKt8lb7-YLmh3cXe2c8XkO6o/view?usp=drive_link</v>
+      </c>
+      <c r="Q267" t="str">
+        <v>https://drive.google.com/file/d/1gUIW3ZmoWKt8lb7-YLmh3cXe2c8XkO6o/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="268">
       <c r="A268" t="str">
@@ -13222,6 +13582,12 @@
       <c r="O268" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (14-3/5)</v>
       </c>
+      <c r="P268" t="str">
+        <v>https://drive.google.com/file/d/1gUIW3ZmoWKt8lb7-YLmh3cXe2c8XkO6o/view?usp=drive_link</v>
+      </c>
+      <c r="Q268" t="str">
+        <v>https://drive.google.com/file/d/1gUIW3ZmoWKt8lb7-YLmh3cXe2c8XkO6o/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="269">
       <c r="A269" t="str">
@@ -13269,6 +13635,12 @@
       <c r="O269" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (14-4/5)</v>
       </c>
+      <c r="P269" t="str">
+        <v>https://drive.google.com/file/d/1gUIW3ZmoWKt8lb7-YLmh3cXe2c8XkO6o/view?usp=drive_link</v>
+      </c>
+      <c r="Q269" t="str">
+        <v>https://drive.google.com/file/d/1gUIW3ZmoWKt8lb7-YLmh3cXe2c8XkO6o/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="270">
       <c r="A270" t="str">
@@ -13316,6 +13688,12 @@
       <c r="O270" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (14-5/5)</v>
       </c>
+      <c r="P270" t="str">
+        <v>https://drive.google.com/file/d/1gUIW3ZmoWKt8lb7-YLmh3cXe2c8XkO6o/view?usp=drive_link</v>
+      </c>
+      <c r="Q270" t="str">
+        <v>https://drive.google.com/file/d/1gUIW3ZmoWKt8lb7-YLmh3cXe2c8XkO6o/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="271">
       <c r="A271" t="str">
@@ -13363,6 +13741,12 @@
       <c r="O271" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (15-1/1)</v>
       </c>
+      <c r="P271" t="str">
+        <v>https://drive.google.com/file/d/1LAPzZrtJ4vSLglxDAanS8u7XSnSEZWLz/view?usp=drive_link</v>
+      </c>
+      <c r="Q271" t="str">
+        <v>https://drive.google.com/file/d/1LAPzZrtJ4vSLglxDAanS8u7XSnSEZWLz/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="272">
       <c r="A272" t="str">
@@ -13410,6 +13794,12 @@
       <c r="O272" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (16-1/1)</v>
       </c>
+      <c r="P272" t="str">
+        <v>https://drive.google.com/file/d/1xYU5dg-p7Fp7vcEbvRLcdEH2Kcv355SC/view?usp=drive_link</v>
+      </c>
+      <c r="Q272" t="str">
+        <v>https://drive.google.com/file/d/1xYU5dg-p7Fp7vcEbvRLcdEH2Kcv355SC/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="str">
@@ -13457,6 +13847,12 @@
       <c r="O273" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (17-1/2)</v>
       </c>
+      <c r="P273" t="str">
+        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+      </c>
+      <c r="Q273" t="str">
+        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="274">
       <c r="A274" t="str">
@@ -13504,6 +13900,12 @@
       <c r="O274" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (17-2/2)</v>
       </c>
+      <c r="P274" t="str">
+        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+      </c>
+      <c r="Q274" t="str">
+        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="275">
       <c r="A275" t="str">
@@ -13551,6 +13953,12 @@
       <c r="O275" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (18-1/2)</v>
       </c>
+      <c r="P275" t="str">
+        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+      </c>
+      <c r="Q275" t="str">
+        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="str">
@@ -13598,6 +14006,12 @@
       <c r="O276" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (18-2/2)</v>
       </c>
+      <c r="P276" t="str">
+        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+      </c>
+      <c r="Q276" t="str">
+        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="str">
@@ -13645,6 +14059,12 @@
       <c r="O277" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (19-1/1)</v>
       </c>
+      <c r="P277" t="str">
+        <v>https://drive.google.com/file/d/1o9-9vXu1-lcc7ZpD1nFG1Jg3m1u0q-jP/view?usp=drive_link</v>
+      </c>
+      <c r="Q277" t="str">
+        <v>https://drive.google.com/file/d/1o9-9vXu1-lcc7ZpD1nFG1Jg3m1u0q-jP/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="278">
       <c r="A278" t="str">
@@ -14397,6 +14817,12 @@
       <c r="O293" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (26-1/2)</v>
       </c>
+      <c r="P293" t="str">
+        <v>https://drive.google.com/file/d/1Q4vzQndJibrlDHeHKA_tvuba478CqoKc/view?usp=drive_link</v>
+      </c>
+      <c r="Q293" t="str">
+        <v>https://drive.google.com/file/d/1Q4vzQndJibrlDHeHKA_tvuba478CqoKc/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="str">
@@ -14444,6 +14870,12 @@
       <c r="O294" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (26-2/2)</v>
       </c>
+      <c r="P294" t="str">
+        <v>https://drive.google.com/file/d/1Q4vzQndJibrlDHeHKA_tvuba478CqoKc/view?usp=drive_link</v>
+      </c>
+      <c r="Q294" t="str">
+        <v>https://drive.google.com/file/d/1Q4vzQndJibrlDHeHKA_tvuba478CqoKc/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="295">
       <c r="A295" t="str">
@@ -15243,6 +15675,12 @@
       <c r="O311" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (29-1/3)</v>
       </c>
+      <c r="P311" t="str">
+        <v>https://drive.google.com/file/d/1kwUGb5m1pAG1CO8kBcaraJx1saRiB2X2/view?usp=drive_link</v>
+      </c>
+      <c r="Q311" t="str">
+        <v>https://drive.google.com/file/d/1kwUGb5m1pAG1CO8kBcaraJx1saRiB2X2/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="str">
@@ -15290,6 +15728,12 @@
       <c r="O312" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (29-2/3)</v>
       </c>
+      <c r="P312" t="str">
+        <v>https://drive.google.com/file/d/1kwUGb5m1pAG1CO8kBcaraJx1saRiB2X2/view?usp=drive_link</v>
+      </c>
+      <c r="Q312" t="str">
+        <v>https://drive.google.com/file/d/1kwUGb5m1pAG1CO8kBcaraJx1saRiB2X2/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="str">
@@ -15337,6 +15781,12 @@
       <c r="O313" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (29-3/3)</v>
       </c>
+      <c r="P313" t="str">
+        <v>https://drive.google.com/file/d/1kwUGb5m1pAG1CO8kBcaraJx1saRiB2X2/view?usp=drive_link</v>
+      </c>
+      <c r="Q313" t="str">
+        <v>https://drive.google.com/file/d/1kwUGb5m1pAG1CO8kBcaraJx1saRiB2X2/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="str">
@@ -15384,6 +15834,12 @@
       <c r="O314" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (30-1/3)</v>
       </c>
+      <c r="P314" t="str">
+        <v>https://drive.google.com/file/d/1FGG2g0tmADlSiukBM-ssFInNmVwzMl4B/view?usp=drive_link</v>
+      </c>
+      <c r="Q314" t="str">
+        <v>https://drive.google.com/file/d/1FGG2g0tmADlSiukBM-ssFInNmVwzMl4B/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="str">
@@ -15431,6 +15887,12 @@
       <c r="O315" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (30-2/3)</v>
       </c>
+      <c r="P315" t="str">
+        <v>https://drive.google.com/file/d/1FGG2g0tmADlSiukBM-ssFInNmVwzMl4B/view?usp=drive_link</v>
+      </c>
+      <c r="Q315" t="str">
+        <v>https://drive.google.com/file/d/1FGG2g0tmADlSiukBM-ssFInNmVwzMl4B/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="316">
       <c r="A316" t="str">
@@ -15478,6 +15940,12 @@
       <c r="O316" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (30-3/3)</v>
       </c>
+      <c r="P316" t="str">
+        <v>https://drive.google.com/file/d/1FGG2g0tmADlSiukBM-ssFInNmVwzMl4B/view?usp=drive_link</v>
+      </c>
+      <c r="Q316" t="str">
+        <v>https://drive.google.com/file/d/1FGG2g0tmADlSiukBM-ssFInNmVwzMl4B/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="317">
       <c r="A317" t="str">
@@ -15619,6 +16087,12 @@
       <c r="O319" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (32-1/1)</v>
       </c>
+      <c r="P319" t="str">
+        <v>https://drive.google.com/file/d/1lIR6N2bcFRHyjLFEjDPHAHsO_IbM-s1G/view?usp=drive_link</v>
+      </c>
+      <c r="Q319" t="str">
+        <v>https://drive.google.com/file/d/1lIR6N2bcFRHyjLFEjDPHAHsO_IbM-s1G/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="320">
       <c r="A320" t="str">
@@ -15666,6 +16140,12 @@
       <c r="O320" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (33-1/8)</v>
       </c>
+      <c r="P320" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
+      <c r="Q320" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="321">
       <c r="A321" t="str">
@@ -15713,6 +16193,12 @@
       <c r="O321" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (33-2/8)</v>
       </c>
+      <c r="P321" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
+      <c r="Q321" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="322">
       <c r="A322" t="str">
@@ -15760,6 +16246,12 @@
       <c r="O322" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (33-3/8)</v>
       </c>
+      <c r="P322" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
+      <c r="Q322" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="323">
       <c r="A323" t="str">
@@ -15807,6 +16299,12 @@
       <c r="O323" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (33-4/8)</v>
       </c>
+      <c r="P323" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
+      <c r="Q323" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="324">
       <c r="A324" t="str">
@@ -15854,6 +16352,12 @@
       <c r="O324" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (33-5/8)</v>
       </c>
+      <c r="P324" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
+      <c r="Q324" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="325">
       <c r="A325" t="str">
@@ -15901,6 +16405,12 @@
       <c r="O325" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (33-6/8)</v>
       </c>
+      <c r="P325" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
+      <c r="Q325" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="326">
       <c r="A326" t="str">
@@ -15948,6 +16458,12 @@
       <c r="O326" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (33-7/8)</v>
       </c>
+      <c r="P326" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
+      <c r="Q326" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="327">
       <c r="A327" t="str">
@@ -15995,6 +16511,12 @@
       <c r="O327" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (33-8/8)</v>
       </c>
+      <c r="P327" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
+      <c r="Q327" t="str">
+        <v>https://drive.google.com/file/d/1gGoEmfJLvV6rJbx-KknmskQ59BBSCfJe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="328">
       <c r="A328" t="str">
@@ -16042,6 +16564,12 @@
       <c r="O328" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (34-1/2)</v>
       </c>
+      <c r="P328" t="str">
+        <v>https://drive.google.com/file/d/1sQXjc7ZdPl8HPtB_lBpHe8iU086ncDjJ/view?usp=drive_link</v>
+      </c>
+      <c r="Q328" t="str">
+        <v>https://drive.google.com/file/d/1sQXjc7ZdPl8HPtB_lBpHe8iU086ncDjJ/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="329">
       <c r="A329" t="str">
@@ -16089,6 +16617,12 @@
       <c r="O329" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (34-2/2)</v>
       </c>
+      <c r="P329" t="str">
+        <v>https://drive.google.com/file/d/1sQXjc7ZdPl8HPtB_lBpHe8iU086ncDjJ/view?usp=drive_link</v>
+      </c>
+      <c r="Q329" t="str">
+        <v>https://drive.google.com/file/d/1sQXjc7ZdPl8HPtB_lBpHe8iU086ncDjJ/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="str">
@@ -16371,6 +16905,12 @@
       <c r="O335" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (36-1/10)</v>
       </c>
+      <c r="P335" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
+      <c r="Q335" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="str">
@@ -16418,6 +16958,12 @@
       <c r="O336" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (36-2/10)</v>
       </c>
+      <c r="P336" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
+      <c r="Q336" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="337">
       <c r="A337" t="str">
@@ -16465,6 +17011,12 @@
       <c r="O337" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (36-3/10)</v>
       </c>
+      <c r="P337" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
+      <c r="Q337" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="str">
@@ -16512,6 +17064,12 @@
       <c r="O338" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (36-4/10)</v>
       </c>
+      <c r="P338" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
+      <c r="Q338" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="str">
@@ -16559,6 +17117,12 @@
       <c r="O339" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (36-5/10)</v>
       </c>
+      <c r="P339" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
+      <c r="Q339" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="340">
       <c r="A340" t="str">
@@ -16606,6 +17170,12 @@
       <c r="O340" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (36-6/10)</v>
       </c>
+      <c r="P340" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
+      <c r="Q340" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="341">
       <c r="A341" t="str">
@@ -16653,6 +17223,12 @@
       <c r="O341" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (36-7/10)</v>
       </c>
+      <c r="P341" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
+      <c r="Q341" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="str">
@@ -16700,6 +17276,12 @@
       <c r="O342" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (36-8/10)</v>
       </c>
+      <c r="P342" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
+      <c r="Q342" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="343">
       <c r="A343" t="str">
@@ -16747,6 +17329,12 @@
       <c r="O343" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (36-9/10)</v>
       </c>
+      <c r="P343" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
+      <c r="Q343" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="344">
       <c r="A344" t="str">
@@ -16794,6 +17382,12 @@
       <c r="O344" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (36-10/10)</v>
       </c>
+      <c r="P344" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
+      <c r="Q344" t="str">
+        <v>https://drive.google.com/file/d/1hsZeSIgZOjd6oIZBCmJ2rf1IE_f8-UmW/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="345">
       <c r="A345" t="str">
@@ -16840,6 +17434,12 @@
       </c>
       <c r="O345" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (37-1/1)</v>
+      </c>
+      <c r="P345" t="str">
+        <v>https://drive.google.com/file/d/16bnMzkcZ4KPDpz-CtHmKLy_DVBAlfTBb/view?usp=drive_link</v>
+      </c>
+      <c r="Q345" t="str">
+        <v>https://drive.google.com/file/d/16bnMzkcZ4KPDpz-CtHmKLy_DVBAlfTBb/view?usp=drive_link</v>
       </c>
     </row>
     <row r="346">

</xml_diff>

<commit_message>
fix(equipment): update image URLs for baby care mannequins (11, 12) and catheterization simulator (144-156)
</commit_message>
<xml_diff>
--- a/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
+++ b/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
@@ -3714,6 +3714,12 @@
       <c r="O68" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (9-1/3)</v>
       </c>
+      <c r="P68" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
+      <c r="Q68" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="str">
@@ -3761,6 +3767,12 @@
       <c r="O69" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (9-2/3)</v>
       </c>
+      <c r="P69" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
+      <c r="Q69" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="str">
@@ -3808,6 +3820,12 @@
       <c r="O70" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (9-3/3)</v>
       </c>
+      <c r="P70" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
+      <c r="Q70" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="str">
@@ -3855,6 +3873,12 @@
       <c r="O71" t="str">
         <v>1-B9701-FA17-65450010004/017-68</v>
       </c>
+      <c r="P71" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
+      <c r="Q71" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="str">
@@ -3902,6 +3926,12 @@
       <c r="O72" t="str">
         <v>1-B9701-FA17-65450010004/018-68</v>
       </c>
+      <c r="P72" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
+      <c r="Q72" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="str">
@@ -3949,6 +3979,12 @@
       <c r="O73" t="str">
         <v>1-B9701-FA17-65450010004/019-68</v>
       </c>
+      <c r="P73" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
+      <c r="Q73" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="str">
@@ -3996,6 +4032,12 @@
       <c r="O74" t="str">
         <v>1-B9701-FA17-65450010004/020-68</v>
       </c>
+      <c r="P74" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
+      <c r="Q74" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="str">
@@ -4043,6 +4085,12 @@
       <c r="O75" t="str">
         <v>1-B9701-FA17-65450010004/021-68</v>
       </c>
+      <c r="P75" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
+      <c r="Q75" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="str">
@@ -4090,6 +4138,12 @@
       <c r="O76" t="str">
         <v>1-B9701-FA17-65450010004/022-68</v>
       </c>
+      <c r="P76" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
+      <c r="Q76" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="str">
@@ -4137,6 +4191,12 @@
       <c r="O77" t="str">
         <v>1-B9701-FA17-65450010004/023-68</v>
       </c>
+      <c r="P77" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
+      <c r="Q77" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="str">
@@ -4184,6 +4244,12 @@
       <c r="O78" t="str">
         <v>1-B9701-FA17-65450010004/024-68</v>
       </c>
+      <c r="P78" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
+      <c r="Q78" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="str">
@@ -4231,6 +4297,12 @@
       <c r="O79" t="str">
         <v>1-B9701-FA17-65450010004/025-68</v>
       </c>
+      <c r="P79" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
+      <c r="Q79" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="str">
@@ -4278,6 +4350,12 @@
       <c r="O80" t="str">
         <v>1-B9701-FA17-65450010004/026-68</v>
       </c>
+      <c r="P80" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
+      <c r="Q80" t="str">
+        <v>https://drive.google.com/file/d/14LvWKWvQuOa_B4OO4QOFRgdj338vXCha/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
@@ -13848,10 +13926,10 @@
         <v>2-B9701-FA17-65450010002/001-67 (17-1/2)</v>
       </c>
       <c r="P273" t="str">
-        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+        <v>https://drive.google.com/file/d/1tuK7VZyzaVF0k8TcPancxcG9ZIVGOVKI/view?usp=drive_link</v>
       </c>
       <c r="Q273" t="str">
-        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+        <v>https://drive.google.com/file/d/1tuK7VZyzaVF0k8TcPancxcG9ZIVGOVKI/view?usp=drive_link</v>
       </c>
     </row>
     <row r="274">
@@ -13901,10 +13979,10 @@
         <v>2-B9701-FA17-65450010002/001-67 (17-2/2)</v>
       </c>
       <c r="P274" t="str">
-        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+        <v>https://drive.google.com/file/d/1tuK7VZyzaVF0k8TcPancxcG9ZIVGOVKI/view?usp=drive_link</v>
       </c>
       <c r="Q274" t="str">
-        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+        <v>https://drive.google.com/file/d/1tuK7VZyzaVF0k8TcPancxcG9ZIVGOVKI/view?usp=drive_link</v>
       </c>
     </row>
     <row r="275">
@@ -13954,10 +14032,10 @@
         <v>2-B9701-FA17-65450010002/001-67 (18-1/2)</v>
       </c>
       <c r="P275" t="str">
-        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+        <v>https://drive.google.com/file/d/1tuK7VZyzaVF0k8TcPancxcG9ZIVGOVKI/view?usp=drive_link</v>
       </c>
       <c r="Q275" t="str">
-        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+        <v>https://drive.google.com/file/d/1tuK7VZyzaVF0k8TcPancxcG9ZIVGOVKI/view?usp=drive_link</v>
       </c>
     </row>
     <row r="276">
@@ -14007,10 +14085,10 @@
         <v>2-B9701-FA17-65450010002/001-67 (18-2/2)</v>
       </c>
       <c r="P276" t="str">
-        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+        <v>https://drive.google.com/file/d/1tuK7VZyzaVF0k8TcPancxcG9ZIVGOVKI/view?usp=drive_link</v>
       </c>
       <c r="Q276" t="str">
-        <v>https://drive.google.com/file/d/1--FrJWzbFfALzPz7mSkJE24U-Nqe7rSB/view?usp=drive_link</v>
+        <v>https://drive.google.com/file/d/1tuK7VZyzaVF0k8TcPancxcG9ZIVGOVKI/view?usp=drive_link</v>
       </c>
     </row>
     <row r="277">

</xml_diff>

<commit_message>
fix(equipment): update image URLs for nasogastric tube simulators (EQ-NG-0001 to 0005, EQ-NG-0011)
</commit_message>
<xml_diff>
--- a/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
+++ b/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
@@ -3479,6 +3479,12 @@
       <c r="O63" t="str">
         <v>1-B9701-FA17-65450010004/012-68</v>
       </c>
+      <c r="P63" t="str">
+        <v>https://drive.google.com/file/d/1Ir_mPIWRqlIZ2YuAT4iKKy2gcWLzhm2E/view?usp=drive_link</v>
+      </c>
+      <c r="Q63" t="str">
+        <v>https://drive.google.com/file/d/1Ir_mPIWRqlIZ2YuAT4iKKy2gcWLzhm2E/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="str">
@@ -3526,6 +3532,12 @@
       <c r="O64" t="str">
         <v>1-B9701-FA17-65450010004/013-68</v>
       </c>
+      <c r="P64" t="str">
+        <v>https://drive.google.com/file/d/1Ir_mPIWRqlIZ2YuAT4iKKy2gcWLzhm2E/view?usp=drive_link</v>
+      </c>
+      <c r="Q64" t="str">
+        <v>https://drive.google.com/file/d/1Ir_mPIWRqlIZ2YuAT4iKKy2gcWLzhm2E/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="str">
@@ -3573,6 +3585,12 @@
       <c r="O65" t="str">
         <v>1-B9701-FA17-65450010004/014-68</v>
       </c>
+      <c r="P65" t="str">
+        <v>https://drive.google.com/file/d/1Ir_mPIWRqlIZ2YuAT4iKKy2gcWLzhm2E/view?usp=drive_link</v>
+      </c>
+      <c r="Q65" t="str">
+        <v>https://drive.google.com/file/d/1Ir_mPIWRqlIZ2YuAT4iKKy2gcWLzhm2E/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="str">
@@ -3620,6 +3638,12 @@
       <c r="O66" t="str">
         <v>1-B9701-FA17-65450010004/015-68</v>
       </c>
+      <c r="P66" t="str">
+        <v>https://drive.google.com/file/d/1Ir_mPIWRqlIZ2YuAT4iKKy2gcWLzhm2E/view?usp=drive_link</v>
+      </c>
+      <c r="Q66" t="str">
+        <v>https://drive.google.com/file/d/1Ir_mPIWRqlIZ2YuAT4iKKy2gcWLzhm2E/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="str">
@@ -3667,6 +3691,12 @@
       <c r="O67" t="str">
         <v>1-B9701-FA17-65450010004/016-68</v>
       </c>
+      <c r="P67" t="str">
+        <v>https://drive.google.com/file/d/1Ir_mPIWRqlIZ2YuAT4iKKy2gcWLzhm2E/view?usp=drive_link</v>
+      </c>
+      <c r="Q67" t="str">
+        <v>https://drive.google.com/file/d/1Ir_mPIWRqlIZ2YuAT4iKKy2gcWLzhm2E/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="str">
@@ -13412,6 +13442,12 @@
       </c>
       <c r="O263" t="str">
         <v>2-B9701-FA17-65450010002/001-67 (8-1/1)</v>
+      </c>
+      <c r="P263" t="str">
+        <v>https://drive.google.com/file/d/1Ir_mPIWRqlIZ2YuAT4iKKy2gcWLzhm2E/view?usp=drive_link</v>
+      </c>
+      <c r="Q263" t="str">
+        <v>https://drive.google.com/file/d/1Ir_mPIWRqlIZ2YuAT4iKKy2gcWLzhm2E/view?usp=drive_link</v>
       </c>
     </row>
     <row r="264">

</xml_diff>

<commit_message>
refactor(equipment): rename EQ-FMS-0001/0002 to EQ-AI-0001/0002, shift existing AI codes, and update suture wound images
</commit_message>
<xml_diff>
--- a/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
+++ b/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
@@ -551,7 +551,7 @@
         <v>จอ LED 40 นิ้ว</v>
       </c>
       <c r="B4" t="str">
-        <v>EQ-AI-0001</v>
+        <v>EQ-AI-0003</v>
       </c>
       <c r="C4" t="str">
         <v>EQUIPMENT</v>
@@ -591,6 +591,12 @@
       </c>
       <c r="O4" t="str">
         <v>1-B9701-FA09-66600010001/003-68</v>
+      </c>
+      <c r="P4" t="str">
+        <v>https://drive.google.com/file/d/160g4PcsX-3XGAXL-EOawSV-chhNloiWr/view?usp=drive_link</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>https://drive.google.com/file/d/160g4PcsX-3XGAXL-EOawSV-chhNloiWr/view?usp=drive_link</v>
       </c>
     </row>
     <row r="5">
@@ -598,7 +604,7 @@
         <v>จอ LED 40 นิ้ว</v>
       </c>
       <c r="B5" t="str">
-        <v>EQ-AI-0002</v>
+        <v>EQ-AI-0004</v>
       </c>
       <c r="C5" t="str">
         <v>EQUIPMENT</v>
@@ -638,6 +644,12 @@
       </c>
       <c r="O5" t="str">
         <v>1-B9701-FA09-66600010001/004-68</v>
+      </c>
+      <c r="P5" t="str">
+        <v>https://drive.google.com/file/d/160g4PcsX-3XGAXL-EOawSV-chhNloiWr/view?usp=drive_link</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>https://drive.google.com/file/d/160g4PcsX-3XGAXL-EOawSV-chhNloiWr/view?usp=drive_link</v>
       </c>
     </row>
     <row r="6">
@@ -2871,16 +2883,16 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>หุ่นฝึกทักษะการพยาบาลขั้นสูง</v>
+        <v>(AI) หุ่นฝึกทักษะการพยาบาลขั้นสูง</v>
       </c>
       <c r="B51" t="str">
-        <v>EQ-FMS-0001</v>
+        <v>EQ-AI-0001</v>
       </c>
       <c r="C51" t="str">
         <v>EQUIPMENT</v>
       </c>
       <c r="D51" t="str">
-        <v>หุ่นฝึกปฏิบัติการ</v>
+        <v>(หุ่น AI) อุปกรณ์จำลองสถานการณ์และหุ่นฝึกปฏิบัติการ</v>
       </c>
       <c r="E51" t="str">
         <v>ตัว</v>
@@ -2915,19 +2927,25 @@
       <c r="O51" t="str">
         <v>1-B9701-FA17-65450010004/001-68</v>
       </c>
+      <c r="P51" t="str">
+        <v>https://drive.google.com/file/d/160g4PcsX-3XGAXL-EOawSV-chhNloiWr/view?usp=drive_link</v>
+      </c>
+      <c r="Q51" t="str">
+        <v>https://drive.google.com/file/d/160g4PcsX-3XGAXL-EOawSV-chhNloiWr/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>หุ่นฝึกทักษะการพยาบาลขั้นสูง</v>
+        <v>(AI) หุ่นฝึกทักษะการพยาบาลขั้นสูง</v>
       </c>
       <c r="B52" t="str">
-        <v>EQ-FMS-0002</v>
+        <v>EQ-AI-0002</v>
       </c>
       <c r="C52" t="str">
         <v>EQUIPMENT</v>
       </c>
       <c r="D52" t="str">
-        <v>หุ่นฝึกปฏิบัติการ</v>
+        <v>(หุ่น AI) อุปกรณ์จำลองสถานการณ์และหุ่นฝึกปฏิบัติการ</v>
       </c>
       <c r="E52" t="str">
         <v>ตัว</v>
@@ -2961,6 +2979,12 @@
       </c>
       <c r="O52" t="str">
         <v>1-B9701-FA17-65450010004/002-68</v>
+      </c>
+      <c r="P52" t="str">
+        <v>https://drive.google.com/file/d/160g4PcsX-3XGAXL-EOawSV-chhNloiWr/view?usp=drive_link</v>
+      </c>
+      <c r="Q52" t="str">
+        <v>https://drive.google.com/file/d/160g4PcsX-3XGAXL-EOawSV-chhNloiWr/view?usp=drive_link</v>
       </c>
     </row>
     <row r="53">
@@ -4986,6 +5010,12 @@
       <c r="O92" t="str">
         <v>1-B9701-FA17-65450010004/037-68</v>
       </c>
+      <c r="P92" t="str">
+        <v>https://drive.google.com/file/d/1Apnn2Cv17dKLqEpoC880iie1yw0h0dWi/view?usp=drive_link</v>
+      </c>
+      <c r="Q92" t="str">
+        <v>https://drive.google.com/file/d/1Apnn2Cv17dKLqEpoC880iie1yw0h0dWi/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="str">
@@ -5033,6 +5063,12 @@
       <c r="O93" t="str">
         <v>1-B9701-FA17-65450010004/038-68</v>
       </c>
+      <c r="P93" t="str">
+        <v>https://drive.google.com/file/d/1Apnn2Cv17dKLqEpoC880iie1yw0h0dWi/view?usp=drive_link</v>
+      </c>
+      <c r="Q93" t="str">
+        <v>https://drive.google.com/file/d/1Apnn2Cv17dKLqEpoC880iie1yw0h0dWi/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="str">
@@ -5080,6 +5116,12 @@
       <c r="O94" t="str">
         <v>1-B9701-FA17-65450010004/039-68</v>
       </c>
+      <c r="P94" t="str">
+        <v>https://drive.google.com/file/d/1Apnn2Cv17dKLqEpoC880iie1yw0h0dWi/view?usp=drive_link</v>
+      </c>
+      <c r="Q94" t="str">
+        <v>https://drive.google.com/file/d/1Apnn2Cv17dKLqEpoC880iie1yw0h0dWi/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="str">
@@ -5127,6 +5169,12 @@
       <c r="O95" t="str">
         <v>1-B9701-FA17-65450010004/040-68</v>
       </c>
+      <c r="P95" t="str">
+        <v>https://drive.google.com/file/d/1Apnn2Cv17dKLqEpoC880iie1yw0h0dWi/view?usp=drive_link</v>
+      </c>
+      <c r="Q95" t="str">
+        <v>https://drive.google.com/file/d/1Apnn2Cv17dKLqEpoC880iie1yw0h0dWi/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="str">
@@ -5174,6 +5222,12 @@
       <c r="O96" t="str">
         <v>1-B9701-FA17-65450010004/041-68</v>
       </c>
+      <c r="P96" t="str">
+        <v>https://drive.google.com/file/d/1zhlhxNTY-rzff8WTB56zfEyAOVqrt6Xe/view?usp=drive_link</v>
+      </c>
+      <c r="Q96" t="str">
+        <v>https://drive.google.com/file/d/1zhlhxNTY-rzff8WTB56zfEyAOVqrt6Xe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="str">
@@ -5221,6 +5275,12 @@
       <c r="O97" t="str">
         <v>1-B9701-FA17-65450010004/042-68</v>
       </c>
+      <c r="P97" t="str">
+        <v>https://drive.google.com/file/d/1zhlhxNTY-rzff8WTB56zfEyAOVqrt6Xe/view?usp=drive_link</v>
+      </c>
+      <c r="Q97" t="str">
+        <v>https://drive.google.com/file/d/1zhlhxNTY-rzff8WTB56zfEyAOVqrt6Xe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="str">
@@ -5268,6 +5328,12 @@
       <c r="O98" t="str">
         <v>1-B9701-FA17-65450010004/043-68</v>
       </c>
+      <c r="P98" t="str">
+        <v>https://drive.google.com/file/d/1zhlhxNTY-rzff8WTB56zfEyAOVqrt6Xe/view?usp=drive_link</v>
+      </c>
+      <c r="Q98" t="str">
+        <v>https://drive.google.com/file/d/1zhlhxNTY-rzff8WTB56zfEyAOVqrt6Xe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="str">
@@ -5315,6 +5381,12 @@
       <c r="O99" t="str">
         <v>1-B9701-FA17-65450010004/044-68</v>
       </c>
+      <c r="P99" t="str">
+        <v>https://drive.google.com/file/d/1zhlhxNTY-rzff8WTB56zfEyAOVqrt6Xe/view?usp=drive_link</v>
+      </c>
+      <c r="Q99" t="str">
+        <v>https://drive.google.com/file/d/1zhlhxNTY-rzff8WTB56zfEyAOVqrt6Xe/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="str">
@@ -7267,6 +7339,12 @@
       <c r="O139" t="str">
         <v>1-B9701-FN17-65450010002/004-68</v>
       </c>
+      <c r="P139" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q139" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="str">
@@ -7314,6 +7392,12 @@
       <c r="O140" t="str">
         <v>1-B9701-FN17-65450010002/005-68</v>
       </c>
+      <c r="P140" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q140" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
@@ -7361,6 +7445,12 @@
       <c r="O141" t="str">
         <v>1-B9701-FN17-65450010002/006-68</v>
       </c>
+      <c r="P141" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q141" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="str">
@@ -7408,6 +7498,12 @@
       <c r="O142" t="str">
         <v>1-B9701-FN17-65450010002/007-68</v>
       </c>
+      <c r="P142" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q142" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="str">
@@ -7455,6 +7551,12 @@
       <c r="O143" t="str">
         <v>1-B9701-FN17-65450010002/008-68</v>
       </c>
+      <c r="P143" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q143" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="str">
@@ -7502,6 +7604,12 @@
       <c r="O144" t="str">
         <v>1-B9701-FN17-65450010002/009-68</v>
       </c>
+      <c r="P144" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q144" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="str">
@@ -7549,6 +7657,12 @@
       <c r="O145" t="str">
         <v>1-B9701-FN17-65450010002/010-68</v>
       </c>
+      <c r="P145" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q145" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="str">
@@ -7596,6 +7710,12 @@
       <c r="O146" t="str">
         <v>1-B9701-FN17-65450010002/011-68</v>
       </c>
+      <c r="P146" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q146" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="str">
@@ -7643,6 +7763,12 @@
       <c r="O147" t="str">
         <v>1-B9701-FN17-65450010002/012-68</v>
       </c>
+      <c r="P147" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q147" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="str">
@@ -7690,6 +7816,12 @@
       <c r="O148" t="str">
         <v>1-B9701-FN17-65450010002/013-68</v>
       </c>
+      <c r="P148" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q148" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="str">
@@ -7737,6 +7869,12 @@
       <c r="O149" t="str">
         <v>1-B9701-FN17-65450010002/014-68</v>
       </c>
+      <c r="P149" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q149" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
@@ -7784,6 +7922,12 @@
       <c r="O150" t="str">
         <v>1-B9701-FN17-65450010002/015-68</v>
       </c>
+      <c r="P150" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q150" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="str">
@@ -7831,6 +7975,12 @@
       <c r="O151" t="str">
         <v>1-B9701-FN17-65450010002/016-68</v>
       </c>
+      <c r="P151" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q151" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="str">
@@ -7878,6 +8028,12 @@
       <c r="O152" t="str">
         <v>1-B9701-FN17-65450010002/017-68</v>
       </c>
+      <c r="P152" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q152" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="str">
@@ -7925,6 +8081,12 @@
       <c r="O153" t="str">
         <v>1-B9701-FN17-65450010002/018-68</v>
       </c>
+      <c r="P153" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q153" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="str">
@@ -7972,6 +8134,12 @@
       <c r="O154" t="str">
         <v>1-B9701-FN17-65450010002/019-68</v>
       </c>
+      <c r="P154" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q154" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="str">
@@ -8019,6 +8187,12 @@
       <c r="O155" t="str">
         <v>1-B9701-FN17-65450010002/020-68</v>
       </c>
+      <c r="P155" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q155" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="str">
@@ -8066,6 +8240,12 @@
       <c r="O156" t="str">
         <v>1-B9701-FN17-65450010002/021-68</v>
       </c>
+      <c r="P156" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q156" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
@@ -8113,6 +8293,12 @@
       <c r="O157" t="str">
         <v>1-B9701-FN17-65450010002/022-68</v>
       </c>
+      <c r="P157" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q157" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="str">
@@ -8160,13 +8346,19 @@
       <c r="O158" t="str">
         <v>1-B9701-FN17-65450010002/023-68</v>
       </c>
+      <c r="P158" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
+      <c r="Q158" t="str">
+        <v>https://drive.google.com/file/d/1NODeU_bXayA8qoaU9lHnnHomnTzKrsxK/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="str">
         <v>แทบเล็ตสำหรับหุ่น AI</v>
       </c>
       <c r="B159" t="str">
-        <v>EQ-AI-0003</v>
+        <v>EQ-AI-0005</v>
       </c>
       <c r="C159" t="str">
         <v>EQUIPMENT</v>
@@ -8213,7 +8405,7 @@
         <v>แทบเล็ตสำหรับหุ่น AI</v>
       </c>
       <c r="B160" t="str">
-        <v>EQ-AI-0004</v>
+        <v>EQ-AI-0006</v>
       </c>
       <c r="C160" t="str">
         <v>EQUIPMENT</v>

</xml_diff>

<commit_message>
refactor(equipment): reorder SIM and FMS items/assets chronologically by received date
</commit_message>
<xml_diff>
--- a/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
+++ b/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
@@ -457,7 +457,7 @@
         <v>Mini PC สำหรับควบคุมหุ่น (SIM MAN)</v>
       </c>
       <c r="B2" t="str">
-        <v>EQ-SIM-0001</v>
+        <v>EQ-SIM-0002</v>
       </c>
       <c r="C2" t="str">
         <v>EQUIPMENT</v>
@@ -504,7 +504,7 @@
         <v>Mini PC สำหรับควบคุมหุ่น (SIM MAN)</v>
       </c>
       <c r="B3" t="str">
-        <v>EQ-SIM-0002</v>
+        <v>EQ-SIM-0003</v>
       </c>
       <c r="C3" t="str">
         <v>EQUIPMENT</v>
@@ -657,7 +657,7 @@
         <v>จอ LED TOUCH Screen 32 นิ้ว (SIM MAN)</v>
       </c>
       <c r="B6" t="str">
-        <v>EQ-SIM-0003</v>
+        <v>EQ-SIM-0004</v>
       </c>
       <c r="C6" t="str">
         <v>EQUIPMENT</v>
@@ -704,7 +704,7 @@
         <v>จอ LED TOUCH Screen 32 นิ้ว (SIM MAN)</v>
       </c>
       <c r="B7" t="str">
-        <v>EQ-SIM-0004</v>
+        <v>EQ-SIM-0005</v>
       </c>
       <c r="C7" t="str">
         <v>EQUIPMENT</v>
@@ -2203,7 +2203,7 @@
         <v>เตียงหุ่น SIM MAN</v>
       </c>
       <c r="B38" t="str">
-        <v>EQ-SIM-0005</v>
+        <v>EQ-SIM-0006</v>
       </c>
       <c r="C38" t="str">
         <v>EQUIPMENT</v>
@@ -2377,10 +2377,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I41" t="str">
-        <v>Amoul</v>
+        <v>Prestan พรีสแตน</v>
       </c>
       <c r="J41" t="str">
-        <v>รุ่นมาตรฐาน (ปีงบ 68)</v>
+        <v>PP AM 100M MS</v>
       </c>
       <c r="K41" t="str">
         <v>4DEM</v>
@@ -2430,10 +2430,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I42" t="str">
-        <v>Amoul</v>
+        <v>Prestan พรีสแตน</v>
       </c>
       <c r="J42" t="str">
-        <v>รุ่นมาตรฐาน (ปีงบ 68)</v>
+        <v>PP AM 100M MS</v>
       </c>
       <c r="K42" t="str">
         <v>4DEM</v>
@@ -2483,10 +2483,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I43" t="str">
-        <v>Amoul</v>
+        <v>Prestan พรีสแตน</v>
       </c>
       <c r="J43" t="str">
-        <v>รุ่นมาตรฐาน (ปีงบ 68)</v>
+        <v>PP AM 100M MS</v>
       </c>
       <c r="K43" t="str">
         <v>4DEM</v>
@@ -2536,10 +2536,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I44" t="str">
-        <v>Amoul</v>
+        <v>Prestan พรีสแตน</v>
       </c>
       <c r="J44" t="str">
-        <v>รุ่นมาตรฐาน (ปีงบ 68)</v>
+        <v>PP AM 100M MS</v>
       </c>
       <c r="K44" t="str">
         <v>4DEM</v>
@@ -2589,10 +2589,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I45" t="str">
-        <v>Amoul</v>
+        <v>Prestan พรีสแตน</v>
       </c>
       <c r="J45" t="str">
-        <v>รุ่นมาตรฐาน (ปีงบ 68)</v>
+        <v>PP AM 100M MS</v>
       </c>
       <c r="K45" t="str">
         <v>4DEM</v>
@@ -5520,10 +5520,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I102" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J102" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K102" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5573,10 +5573,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I103" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J103" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K103" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5626,10 +5626,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I104" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J104" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K104" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5679,10 +5679,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I105" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J105" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K105" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5732,10 +5732,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I106" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J106" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K106" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5785,10 +5785,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I107" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J107" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K107" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5838,10 +5838,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I108" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J108" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K108" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5891,10 +5891,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I109" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J109" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K109" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5944,10 +5944,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I110" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J110" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K110" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -5997,10 +5997,10 @@
         <v>2025-08-19</v>
       </c>
       <c r="I111" t="str">
-        <v>Nasco Life/form</v>
+        <v>อัพไรท์ ซิมมูเลชั่น</v>
       </c>
       <c r="J111" t="str">
-        <v>LF01043</v>
+        <v>800-816</v>
       </c>
       <c r="K111" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -6499,7 +6499,7 @@
         <v>SIM MAN</v>
       </c>
       <c r="B122" t="str">
-        <v>EQ-SIM-0006</v>
+        <v>EQ-SIM-0007</v>
       </c>
       <c r="C122" t="str">
         <v>EQUIPMENT</v>
@@ -8382,7 +8382,7 @@
         <v>Apple</v>
       </c>
       <c r="J159" t="str">
-        <v>iPad (Alex AI)</v>
+        <v>(Alex AI)</v>
       </c>
       <c r="K159" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -8429,7 +8429,7 @@
         <v>Apple</v>
       </c>
       <c r="J160" t="str">
-        <v>iPad (Alex AI)</v>
+        <v>(Alex AI)</v>
       </c>
       <c r="K160" t="str">
         <v>บริษัท อัพไรท์ ซิมมูเลชั่น  จำกัด</v>
@@ -10447,10 +10447,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I203" t="str">
-        <v>4DEM</v>
+        <v>เตียงเฟาร์เลอร์ 2 ไกร์</v>
       </c>
       <c r="J203" t="str">
-        <v>ไฟฟ้า 2 ไกร์ ราวสไลด์</v>
+        <v>แบบ ดิจิตอล</v>
       </c>
       <c r="K203" t="str">
         <v>4DEM</v>
@@ -10497,7 +10497,7 @@
         <v>4DEM</v>
       </c>
       <c r="J204" t="str">
-        <v>รุ่นมาตรฐาน</v>
+        <v>หุ่น SIM MAN Gaumard Scientific</v>
       </c>
       <c r="K204" t="str">
         <v>4DEM</v>
@@ -10550,7 +10550,7 @@
         <v>4DEM</v>
       </c>
       <c r="J205" t="str">
-        <v>รุ่นมาตรฐาน</v>
+        <v>Qube AVPro</v>
       </c>
       <c r="K205" t="str">
         <v>4DEM</v>
@@ -10594,10 +10594,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I206" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J206" t="str">
-        <v>P93-Male</v>
+        <v>60850</v>
       </c>
       <c r="K206" t="str">
         <v>4DEM</v>
@@ -10647,10 +10647,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I207" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J207" t="str">
-        <v>P93-Male</v>
+        <v>60850</v>
       </c>
       <c r="K207" t="str">
         <v>4DEM</v>
@@ -10700,10 +10700,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I208" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J208" t="str">
-        <v>P93-Male</v>
+        <v>60850</v>
       </c>
       <c r="K208" t="str">
         <v>4DEM</v>
@@ -10753,10 +10753,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I209" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J209" t="str">
-        <v>P93-Male</v>
+        <v>60850</v>
       </c>
       <c r="K209" t="str">
         <v>4DEM</v>
@@ -10806,10 +10806,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I210" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J210" t="str">
-        <v>P93-Male</v>
+        <v>60850</v>
       </c>
       <c r="K210" t="str">
         <v>4DEM</v>
@@ -10859,10 +10859,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I211" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J211" t="str">
-        <v>P93-Female</v>
+        <v>60851</v>
       </c>
       <c r="K211" t="str">
         <v>4DEM</v>
@@ -10912,10 +10912,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I212" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J212" t="str">
-        <v>P93-Female</v>
+        <v>60851</v>
       </c>
       <c r="K212" t="str">
         <v>4DEM</v>
@@ -10965,10 +10965,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I213" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J213" t="str">
-        <v>P93-Female</v>
+        <v>60851</v>
       </c>
       <c r="K213" t="str">
         <v>4DEM</v>
@@ -11018,10 +11018,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I214" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J214" t="str">
-        <v>P93-Female</v>
+        <v>60851</v>
       </c>
       <c r="K214" t="str">
         <v>4DEM</v>
@@ -11071,10 +11071,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I215" t="str">
-        <v>3B Scientific</v>
+        <v>Limbs &amp; Things</v>
       </c>
       <c r="J215" t="str">
-        <v>P93-Female</v>
+        <v>60851</v>
       </c>
       <c r="K215" t="str">
         <v>4DEM</v>
@@ -11124,10 +11124,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I216" t="str">
-        <v>4DEM</v>
+        <v>KOKEN</v>
       </c>
       <c r="J216" t="str">
-        <v>รุ่นมาตรฐาน</v>
+        <v>LM-097B</v>
       </c>
       <c r="K216" t="str">
         <v>4DEM</v>
@@ -11177,10 +11177,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I217" t="str">
-        <v>4DEM</v>
+        <v>KOKEN</v>
       </c>
       <c r="J217" t="str">
-        <v>รุ่นมาตรฐาน</v>
+        <v>LM-097B</v>
       </c>
       <c r="K217" t="str">
         <v>4DEM</v>
@@ -11230,10 +11230,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I218" t="str">
-        <v>4DEM</v>
+        <v>KOKEN</v>
       </c>
       <c r="J218" t="str">
-        <v>รุ่นมาตรฐาน</v>
+        <v>LM-097B</v>
       </c>
       <c r="K218" t="str">
         <v>4DEM</v>
@@ -11283,10 +11283,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I219" t="str">
-        <v>4DEM</v>
+        <v>KOKEN</v>
       </c>
       <c r="J219" t="str">
-        <v>รุ่นมาตรฐาน</v>
+        <v>LM-097B</v>
       </c>
       <c r="K219" t="str">
         <v>4DEM</v>
@@ -11336,10 +11336,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I220" t="str">
-        <v>4DEM</v>
+        <v>KOKEN</v>
       </c>
       <c r="J220" t="str">
-        <v>รุ่นมาตรฐาน</v>
+        <v>LM-097B</v>
       </c>
       <c r="K220" t="str">
         <v>4DEM</v>
@@ -11365,16 +11365,16 @@
     </row>
     <row r="221">
       <c r="A221" t="str">
-        <v>หุ่นจำลองผู้ใหญ่</v>
+        <v>SIM MAN</v>
       </c>
       <c r="B221" t="str">
-        <v>EQ-FMS-0003</v>
+        <v>EQ-SIM-0001</v>
       </c>
       <c r="C221" t="str">
         <v>EQUIPMENT</v>
       </c>
       <c r="D221" t="str">
-        <v>หุ่นฝึกปฏิบัติการ</v>
+        <v>(SIM MAN) อุปกรณ์จำลองสถานการณ์และหุ่นฝึกปฏิบัติการ</v>
       </c>
       <c r="E221" t="str">
         <v>ชุด</v>
@@ -11389,10 +11389,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I221" t="str">
-        <v>3B Scientific</v>
+        <v>Gaumard Scientific</v>
       </c>
       <c r="J221" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>S3201.PK</v>
       </c>
       <c r="K221" t="str">
         <v>4DEM</v>
@@ -11654,10 +11654,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I226" t="str">
-        <v>Nasco Life/form</v>
+        <v>Koken</v>
       </c>
       <c r="J226" t="str">
-        <v>LF00698 Venipuncture Arm</v>
+        <v>LM-028</v>
       </c>
       <c r="K226" t="str">
         <v>4DEM</v>
@@ -11707,10 +11707,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I227" t="str">
-        <v>Nasco Life/form</v>
+        <v>Koken</v>
       </c>
       <c r="J227" t="str">
-        <v>LF00698 Venipuncture Arm</v>
+        <v>LM-028</v>
       </c>
       <c r="K227" t="str">
         <v>4DEM</v>
@@ -11760,10 +11760,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I228" t="str">
-        <v>Nasco Life/form</v>
+        <v>Koken</v>
       </c>
       <c r="J228" t="str">
-        <v>LF00698 Venipuncture Arm</v>
+        <v>LM-028</v>
       </c>
       <c r="K228" t="str">
         <v>4DEM</v>
@@ -11813,10 +11813,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I229" t="str">
-        <v>Nasco Life/form</v>
+        <v>Koken</v>
       </c>
       <c r="J229" t="str">
-        <v>LF00698 Venipuncture Arm</v>
+        <v>LM-028</v>
       </c>
       <c r="K229" t="str">
         <v>4DEM</v>
@@ -11866,10 +11866,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I230" t="str">
-        <v>Nasco Life/form</v>
+        <v>Koken</v>
       </c>
       <c r="J230" t="str">
-        <v>LF00698 Venipuncture Arm</v>
+        <v>LM-028</v>
       </c>
       <c r="K230" t="str">
         <v>4DEM</v>
@@ -11919,10 +11919,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I231" t="str">
-        <v>Nasco Life/form</v>
+        <v>Koken</v>
       </c>
       <c r="J231" t="str">
-        <v>LF00698 Venipuncture Arm</v>
+        <v>LM-028</v>
       </c>
       <c r="K231" t="str">
         <v>4DEM</v>
@@ -11972,10 +11972,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I232" t="str">
-        <v>Nasco Life/form</v>
+        <v>Koken</v>
       </c>
       <c r="J232" t="str">
-        <v>LF00698 Venipuncture Arm</v>
+        <v>LM-028</v>
       </c>
       <c r="K232" t="str">
         <v>4DEM</v>
@@ -12025,10 +12025,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I233" t="str">
-        <v>3B Scientific</v>
+        <v>Nasco Healthcare</v>
       </c>
       <c r="J233" t="str">
-        <v>P100 Wound Care</v>
+        <v>LF00929U</v>
       </c>
       <c r="K233" t="str">
         <v>4DEM</v>
@@ -12078,10 +12078,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I234" t="str">
-        <v>3B Scientific</v>
+        <v>Nasco Healthcare</v>
       </c>
       <c r="J234" t="str">
-        <v>P100 Wound Care</v>
+        <v>LF00929U</v>
       </c>
       <c r="K234" t="str">
         <v>4DEM</v>
@@ -12131,10 +12131,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I235" t="str">
-        <v>3B Scientific</v>
+        <v>Nasco Healthcare</v>
       </c>
       <c r="J235" t="str">
-        <v>P100 Wound Care</v>
+        <v>LF00929U</v>
       </c>
       <c r="K235" t="str">
         <v>4DEM</v>
@@ -12184,10 +12184,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I236" t="str">
-        <v>3B Scientific</v>
+        <v>Nasco Healthcare</v>
       </c>
       <c r="J236" t="str">
-        <v>P100 Wound Care</v>
+        <v>LF00929U</v>
       </c>
       <c r="K236" t="str">
         <v>4DEM</v>
@@ -12237,10 +12237,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I237" t="str">
-        <v>3B Scientific</v>
+        <v>Nasco Healthcare</v>
       </c>
       <c r="J237" t="str">
-        <v>P100 Wound Care</v>
+        <v>LF00929U</v>
       </c>
       <c r="K237" t="str">
         <v>4DEM</v>
@@ -12290,10 +12290,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I238" t="str">
-        <v>Koken</v>
+        <v>4DEM</v>
       </c>
       <c r="J238" t="str">
-        <v>M155-Wearable</v>
+        <v>L-IMD</v>
       </c>
       <c r="K238" t="str">
         <v>4DEM</v>
@@ -12343,10 +12343,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I239" t="str">
-        <v>Koken</v>
+        <v>4DEM</v>
       </c>
       <c r="J239" t="str">
-        <v>M155-Wearable</v>
+        <v>L-IMD</v>
       </c>
       <c r="K239" t="str">
         <v>4DEM</v>
@@ -12396,10 +12396,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I240" t="str">
-        <v>Koken</v>
+        <v>4DEM</v>
       </c>
       <c r="J240" t="str">
-        <v>M155-Wearable</v>
+        <v>L-IMD</v>
       </c>
       <c r="K240" t="str">
         <v>4DEM</v>
@@ -12449,10 +12449,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I241" t="str">
-        <v>Koken</v>
+        <v>4DEM</v>
       </c>
       <c r="J241" t="str">
-        <v>M155-Wearable</v>
+        <v>L-IMD</v>
       </c>
       <c r="K241" t="str">
         <v>4DEM</v>
@@ -12502,10 +12502,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I242" t="str">
-        <v>Koken</v>
+        <v>4DEM</v>
       </c>
       <c r="J242" t="str">
-        <v>M155-Wearable</v>
+        <v>L-IMD</v>
       </c>
       <c r="K242" t="str">
         <v>4DEM</v>
@@ -12534,7 +12534,7 @@
         <v>หุ่นฝึกปฏิบัติการพยาบาลพื้นฐาน (ชาย)</v>
       </c>
       <c r="B243" t="str">
-        <v>EQ-FMS-0004</v>
+        <v>EQ-FMS-0007</v>
       </c>
       <c r="C243" t="str">
         <v>EQUIPMENT</v>
@@ -12555,10 +12555,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I243" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J243" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1M</v>
       </c>
       <c r="K243" t="str">
         <v>4DEM</v>
@@ -12587,7 +12587,7 @@
         <v>หุ่นฝึกปฏิบัติการพยาบาลพื้นฐาน (ชาย)</v>
       </c>
       <c r="B244" t="str">
-        <v>EQ-FMS-0005</v>
+        <v>EQ-FMS-0008</v>
       </c>
       <c r="C244" t="str">
         <v>EQUIPMENT</v>
@@ -12608,10 +12608,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I244" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J244" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1M</v>
       </c>
       <c r="K244" t="str">
         <v>4DEM</v>
@@ -12640,7 +12640,7 @@
         <v>หุ่นฝึกปฏิบัติการพยาบาลพื้นฐาน (ชาย)</v>
       </c>
       <c r="B245" t="str">
-        <v>EQ-FMS-0006</v>
+        <v>EQ-FMS-0009</v>
       </c>
       <c r="C245" t="str">
         <v>EQUIPMENT</v>
@@ -12661,10 +12661,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I245" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J245" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1M</v>
       </c>
       <c r="K245" t="str">
         <v>4DEM</v>
@@ -12693,7 +12693,7 @@
         <v>หุ่นฝึกปฏิบัติการพยาบาลพื้นฐาน (ชาย)</v>
       </c>
       <c r="B246" t="str">
-        <v>EQ-FMS-0007</v>
+        <v>EQ-FMS-0010</v>
       </c>
       <c r="C246" t="str">
         <v>EQUIPMENT</v>
@@ -12714,10 +12714,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I246" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J246" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1M</v>
       </c>
       <c r="K246" t="str">
         <v>4DEM</v>
@@ -12746,7 +12746,7 @@
         <v>หุ่นฝึกปฏิบัติการพยาบาลพื้นฐาน (ชาย)</v>
       </c>
       <c r="B247" t="str">
-        <v>EQ-FMS-0008</v>
+        <v>EQ-FMS-0011</v>
       </c>
       <c r="C247" t="str">
         <v>EQUIPMENT</v>
@@ -12767,10 +12767,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I247" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J247" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1M</v>
       </c>
       <c r="K247" t="str">
         <v>4DEM</v>
@@ -12799,7 +12799,7 @@
         <v>หุ่นฝึกปฏิบัติการพยาบาลพื้นฐาน (หญิง)</v>
       </c>
       <c r="B248" t="str">
-        <v>EQ-FMS-0009</v>
+        <v>EQ-FMS-0012</v>
       </c>
       <c r="C248" t="str">
         <v>EQUIPMENT</v>
@@ -12820,10 +12820,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I248" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J248" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1F</v>
       </c>
       <c r="K248" t="str">
         <v>4DEM</v>
@@ -12852,7 +12852,7 @@
         <v>หุ่นฝึกปฏิบัติการพยาบาลพื้นฐาน (หญิง)</v>
       </c>
       <c r="B249" t="str">
-        <v>EQ-FMS-0010</v>
+        <v>EQ-FMS-0013</v>
       </c>
       <c r="C249" t="str">
         <v>EQUIPMENT</v>
@@ -12873,10 +12873,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I249" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J249" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1F</v>
       </c>
       <c r="K249" t="str">
         <v>4DEM</v>
@@ -12905,7 +12905,7 @@
         <v>หุ่นฝึกปฏิบัติการพยาบาลพื้นฐาน (หญิง)</v>
       </c>
       <c r="B250" t="str">
-        <v>EQ-FMS-0011</v>
+        <v>EQ-FMS-0014</v>
       </c>
       <c r="C250" t="str">
         <v>EQUIPMENT</v>
@@ -12926,10 +12926,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I250" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J250" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1F</v>
       </c>
       <c r="K250" t="str">
         <v>4DEM</v>
@@ -12958,7 +12958,7 @@
         <v>หุ่นฝึกปฏิบัติการพยาบาลพื้นฐาน (หญิง)</v>
       </c>
       <c r="B251" t="str">
-        <v>EQ-FMS-0012</v>
+        <v>EQ-FMS-0015</v>
       </c>
       <c r="C251" t="str">
         <v>EQUIPMENT</v>
@@ -12979,10 +12979,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I251" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J251" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1F</v>
       </c>
       <c r="K251" t="str">
         <v>4DEM</v>
@@ -13011,7 +13011,7 @@
         <v>หุ่นฝึกปฏิบัติการพยาบาลพื้นฐาน (หญิง)</v>
       </c>
       <c r="B252" t="str">
-        <v>EQ-FMS-0013</v>
+        <v>EQ-FMS-0016</v>
       </c>
       <c r="C252" t="str">
         <v>EQUIPMENT</v>
@@ -13032,10 +13032,10 @@
         <v>2025-05-01</v>
       </c>
       <c r="I252" t="str">
-        <v>3B Scientific</v>
+        <v>CLA Nursing Doll</v>
       </c>
       <c r="J252" t="str">
-        <v>Nursing Manikin Standard</v>
+        <v>CLA 1F</v>
       </c>
       <c r="K252" t="str">
         <v>4DEM</v>
@@ -13276,7 +13276,7 @@
         <v>หุ่นฝึกทักษะการพยาบาลผู้ใหญ่</v>
       </c>
       <c r="B257" t="str">
-        <v>EQ-FMS-0014</v>
+        <v>EQ-FMS-0001</v>
       </c>
       <c r="C257" t="str">
         <v>EQUIPMENT</v>
@@ -13329,7 +13329,7 @@
         <v>หุ่นฝึกทักษะการพยาบาลผู้ใหญ่</v>
       </c>
       <c r="B258" t="str">
-        <v>EQ-FMS-0015</v>
+        <v>EQ-FMS-0002</v>
       </c>
       <c r="C258" t="str">
         <v>EQUIPMENT</v>
@@ -13382,7 +13382,7 @@
         <v>หุ่นฝึกทักษะการพยาบาลผู้ใหญ่</v>
       </c>
       <c r="B259" t="str">
-        <v>EQ-FMS-0016</v>
+        <v>EQ-FMS-0003</v>
       </c>
       <c r="C259" t="str">
         <v>EQUIPMENT</v>
@@ -13435,7 +13435,7 @@
         <v>หุ่นฝึกทักษะการพยาบาลผู้ใหญ่</v>
       </c>
       <c r="B260" t="str">
-        <v>EQ-FMS-0017</v>
+        <v>EQ-FMS-0004</v>
       </c>
       <c r="C260" t="str">
         <v>EQUIPMENT</v>
@@ -13488,7 +13488,7 @@
         <v>หุ่นฝึกทักษะการพยาบาลผู้ใหญ่</v>
       </c>
       <c r="B261" t="str">
-        <v>EQ-FMS-0018</v>
+        <v>EQ-FMS-0005</v>
       </c>
       <c r="C261" t="str">
         <v>EQUIPMENT</v>
@@ -13541,7 +13541,7 @@
         <v>หุ่นฝึกทักษะการพยาบาลผู้ใหญ่</v>
       </c>
       <c r="B262" t="str">
-        <v>EQ-FMS-0019</v>
+        <v>EQ-FMS-0006</v>
       </c>
       <c r="C262" t="str">
         <v>EQUIPMENT</v>
@@ -15376,7 +15376,7 @@
         <v>ตู้ข้างเตียง</v>
       </c>
       <c r="B299" t="str">
-        <v>EQ-BED-0042</v>
+        <v>EQ-BED-0041</v>
       </c>
       <c r="C299" t="str">
         <v>EQUIPMENT</v>
@@ -18646,7 +18646,7 @@
         <v>หูฟังแพทย์แบบ 2 ทาง</v>
       </c>
       <c r="B365" t="str">
-        <v>EQ-MED-0017</v>
+        <v>EQ-MED-0018</v>
       </c>
       <c r="C365" t="str">
         <v>EQUIPMENT</v>

</xml_diff>

<commit_message>
feat(equipment): update image URLs for SAM simulators (EQ-SAM-0001 to 0010)
</commit_message>
<xml_diff>
--- a/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
+++ b/ข้อมูลครุภัณฑ์/Template_Items_and_Assets_v3.updated.xlsx
@@ -6070,6 +6070,12 @@
       <c r="O112" t="str">
         <v>1-B9701-FA17-65450010004/055-68</v>
       </c>
+      <c r="P112" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
+      <c r="Q112" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="str">
@@ -6117,6 +6123,12 @@
       <c r="O113" t="str">
         <v>1-B9701-FA17-65450010004/056-68</v>
       </c>
+      <c r="P113" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
+      <c r="Q113" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="str">
@@ -6164,6 +6176,12 @@
       <c r="O114" t="str">
         <v>1-B9701-FA17-65450010004/057-68</v>
       </c>
+      <c r="P114" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
+      <c r="Q114" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="str">
@@ -6211,6 +6229,12 @@
       <c r="O115" t="str">
         <v>1-B9701-FA17-65450010004/058-68</v>
       </c>
+      <c r="P115" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
+      <c r="Q115" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="str">
@@ -6258,6 +6282,12 @@
       <c r="O116" t="str">
         <v>1-B9701-FA17-65450010004/059-68</v>
       </c>
+      <c r="P116" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
+      <c r="Q116" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="str">
@@ -6305,6 +6335,12 @@
       <c r="O117" t="str">
         <v>1-B9701-FA17-65450010004/060-68</v>
       </c>
+      <c r="P117" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
+      <c r="Q117" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="str">
@@ -6352,6 +6388,12 @@
       <c r="O118" t="str">
         <v>1-B9701-FA17-65450010004/061-68</v>
       </c>
+      <c r="P118" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
+      <c r="Q118" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
@@ -6399,6 +6441,12 @@
       <c r="O119" t="str">
         <v>1-B9701-FA17-65450010004/062-68</v>
       </c>
+      <c r="P119" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
+      <c r="Q119" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="str">
@@ -6446,6 +6494,12 @@
       <c r="O120" t="str">
         <v>1-B9701-FA17-65450010004/063-68</v>
       </c>
+      <c r="P120" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
+      <c r="Q120" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="str">
@@ -6492,6 +6546,12 @@
       </c>
       <c r="O121" t="str">
         <v>1-B9701-FA17-65450010004/064-68</v>
+      </c>
+      <c r="P121" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
+      </c>
+      <c r="Q121" t="str">
+        <v>https://drive.google.com/file/d/1LI1x5YY8n31UAw8_Z4AJmhrtLtEvQBmN/view?usp=drive_link</v>
       </c>
     </row>
     <row r="122">

</xml_diff>